<commit_message>
Step3 코드 생성, RULE.md 업데이트 (2026-03-03)
</commit_message>
<xml_diff>
--- a/레포트 양식 기준/파워마스터_20260202_507BWS_호기_(M006161)_OverHaul 작업 件.xlsx
+++ b/레포트 양식 기준/파워마스터_20260202_507BWS_호기_(M006161)_OverHaul 작업 件.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\정동교\문서 자동화 TEST\커서 바이브코딩 자동화 관련\레포트 양식 기준\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9197EDC7-55D4-41F4-B973-CF8682CF2C9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{136BAC0D-A34D-4419-9A65-537C4CFA2BF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="748" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="90">
   <si>
     <t>3. 조치내용</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -931,10 +931,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>사량</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>이전
 교체</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1446,6 +1442,258 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="9" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="9" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="181" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1455,51 +1703,6 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="179" fontId="9" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1507,213 +1710,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="179" fontId="9" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="181" fontId="13" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="9" fillId="3" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="180" fontId="9" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -8558,21 +8554,21 @@
   <sheetData>
     <row r="2" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F2" s="2"/>
-      <c r="S2" s="42" t="s">
+      <c r="S2" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="T2" s="42"/>
-      <c r="U2" s="42"/>
-      <c r="V2" s="42" t="s">
+      <c r="T2" s="65"/>
+      <c r="U2" s="65"/>
+      <c r="V2" s="65" t="s">
         <v>5</v>
       </c>
-      <c r="W2" s="42"/>
-      <c r="X2" s="42"/>
-      <c r="Y2" s="42" t="s">
+      <c r="W2" s="65"/>
+      <c r="X2" s="65"/>
+      <c r="Y2" s="65" t="s">
         <v>6</v>
       </c>
-      <c r="Z2" s="42"/>
-      <c r="AA2" s="42"/>
+      <c r="Z2" s="65"/>
+      <c r="AA2" s="65"/>
     </row>
     <row r="3" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F3" s="4" t="s">
@@ -8590,15 +8586,15 @@
       <c r="P3" s="6"/>
       <c r="Q3" s="6"/>
       <c r="R3" s="6"/>
-      <c r="S3" s="42"/>
-      <c r="T3" s="42"/>
-      <c r="U3" s="42"/>
-      <c r="V3" s="42"/>
-      <c r="W3" s="42"/>
-      <c r="X3" s="42"/>
-      <c r="Y3" s="42"/>
-      <c r="Z3" s="42"/>
-      <c r="AA3" s="42"/>
+      <c r="S3" s="65"/>
+      <c r="T3" s="65"/>
+      <c r="U3" s="65"/>
+      <c r="V3" s="65"/>
+      <c r="W3" s="65"/>
+      <c r="X3" s="65"/>
+      <c r="Y3" s="65"/>
+      <c r="Z3" s="65"/>
+      <c r="AA3" s="65"/>
     </row>
     <row r="4" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F4" s="4" t="s">
@@ -8616,17 +8612,17 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="69" t="s">
+      <c r="S4" s="66" t="s">
         <v>42</v>
       </c>
-      <c r="T4" s="70"/>
-      <c r="U4" s="70"/>
-      <c r="V4" s="69"/>
-      <c r="W4" s="70"/>
-      <c r="X4" s="75"/>
-      <c r="Y4" s="78"/>
-      <c r="Z4" s="78"/>
-      <c r="AA4" s="78"/>
+      <c r="T4" s="67"/>
+      <c r="U4" s="67"/>
+      <c r="V4" s="66"/>
+      <c r="W4" s="67"/>
+      <c r="X4" s="72"/>
+      <c r="Y4" s="75"/>
+      <c r="Z4" s="75"/>
+      <c r="AA4" s="75"/>
     </row>
     <row r="5" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="I5" s="6"/>
@@ -8635,64 +8631,64 @@
       <c r="L5" s="6"/>
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
-      <c r="S5" s="71"/>
-      <c r="T5" s="72"/>
-      <c r="U5" s="72"/>
-      <c r="V5" s="71"/>
-      <c r="W5" s="72"/>
-      <c r="X5" s="76"/>
-      <c r="Y5" s="78"/>
-      <c r="Z5" s="78"/>
-      <c r="AA5" s="78"/>
+      <c r="S5" s="68"/>
+      <c r="T5" s="69"/>
+      <c r="U5" s="69"/>
+      <c r="V5" s="68"/>
+      <c r="W5" s="69"/>
+      <c r="X5" s="73"/>
+      <c r="Y5" s="75"/>
+      <c r="Z5" s="75"/>
+      <c r="AA5" s="75"/>
     </row>
     <row r="6" spans="2:39" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="79" t="s">
+      <c r="B6" s="76" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="79"/>
-      <c r="D6" s="79"/>
-      <c r="E6" s="79"/>
-      <c r="F6" s="79"/>
-      <c r="G6" s="79"/>
-      <c r="H6" s="79"/>
-      <c r="I6" s="79"/>
-      <c r="J6" s="79"/>
-      <c r="K6" s="79"/>
-      <c r="L6" s="79"/>
-      <c r="M6" s="79"/>
-      <c r="N6" s="79"/>
-      <c r="O6" s="79"/>
-      <c r="P6" s="79"/>
-      <c r="Q6" s="79"/>
-      <c r="R6" s="79"/>
-      <c r="S6" s="73"/>
-      <c r="T6" s="74"/>
-      <c r="U6" s="74"/>
-      <c r="V6" s="73"/>
-      <c r="W6" s="74"/>
-      <c r="X6" s="77"/>
-      <c r="Y6" s="78"/>
-      <c r="Z6" s="78"/>
-      <c r="AA6" s="78"/>
+      <c r="C6" s="76"/>
+      <c r="D6" s="76"/>
+      <c r="E6" s="76"/>
+      <c r="F6" s="76"/>
+      <c r="G6" s="76"/>
+      <c r="H6" s="76"/>
+      <c r="I6" s="76"/>
+      <c r="J6" s="76"/>
+      <c r="K6" s="76"/>
+      <c r="L6" s="76"/>
+      <c r="M6" s="76"/>
+      <c r="N6" s="76"/>
+      <c r="O6" s="76"/>
+      <c r="P6" s="76"/>
+      <c r="Q6" s="76"/>
+      <c r="R6" s="76"/>
+      <c r="S6" s="70"/>
+      <c r="T6" s="71"/>
+      <c r="U6" s="71"/>
+      <c r="V6" s="70"/>
+      <c r="W6" s="71"/>
+      <c r="X6" s="74"/>
+      <c r="Y6" s="75"/>
+      <c r="Z6" s="75"/>
+      <c r="AA6" s="75"/>
     </row>
     <row r="7" spans="2:39" ht="3" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="79"/>
-      <c r="C7" s="79"/>
-      <c r="D7" s="79"/>
-      <c r="E7" s="79"/>
-      <c r="F7" s="79"/>
-      <c r="G7" s="79"/>
-      <c r="H7" s="79"/>
-      <c r="I7" s="79"/>
-      <c r="J7" s="79"/>
-      <c r="K7" s="79"/>
-      <c r="L7" s="79"/>
-      <c r="M7" s="79"/>
-      <c r="N7" s="79"/>
-      <c r="O7" s="79"/>
-      <c r="P7" s="79"/>
-      <c r="Q7" s="79"/>
-      <c r="R7" s="79"/>
+      <c r="B7" s="76"/>
+      <c r="C7" s="76"/>
+      <c r="D7" s="76"/>
+      <c r="E7" s="76"/>
+      <c r="F7" s="76"/>
+      <c r="G7" s="76"/>
+      <c r="H7" s="76"/>
+      <c r="I7" s="76"/>
+      <c r="J7" s="76"/>
+      <c r="K7" s="76"/>
+      <c r="L7" s="76"/>
+      <c r="M7" s="76"/>
+      <c r="N7" s="76"/>
+      <c r="O7" s="76"/>
+      <c r="P7" s="76"/>
+      <c r="Q7" s="76"/>
+      <c r="R7" s="76"/>
       <c r="S7" s="8"/>
       <c r="T7" s="8"/>
       <c r="U7" s="8"/>
@@ -8704,34 +8700,34 @@
       <c r="AA7" s="7"/>
     </row>
     <row r="8" spans="2:39" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="79"/>
-      <c r="C8" s="79"/>
-      <c r="D8" s="79"/>
-      <c r="E8" s="79"/>
-      <c r="F8" s="79"/>
-      <c r="G8" s="79"/>
-      <c r="H8" s="79"/>
-      <c r="I8" s="79"/>
-      <c r="J8" s="79"/>
-      <c r="K8" s="79"/>
-      <c r="L8" s="79"/>
-      <c r="M8" s="79"/>
-      <c r="N8" s="79"/>
-      <c r="O8" s="79"/>
-      <c r="P8" s="79"/>
-      <c r="Q8" s="79"/>
-      <c r="R8" s="79"/>
-      <c r="S8" s="63" t="s">
+      <c r="B8" s="76"/>
+      <c r="C8" s="76"/>
+      <c r="D8" s="76"/>
+      <c r="E8" s="76"/>
+      <c r="F8" s="76"/>
+      <c r="G8" s="76"/>
+      <c r="H8" s="76"/>
+      <c r="I8" s="76"/>
+      <c r="J8" s="76"/>
+      <c r="K8" s="76"/>
+      <c r="L8" s="76"/>
+      <c r="M8" s="76"/>
+      <c r="N8" s="76"/>
+      <c r="O8" s="76"/>
+      <c r="P8" s="76"/>
+      <c r="Q8" s="76"/>
+      <c r="R8" s="76"/>
+      <c r="S8" s="77" t="s">
         <v>8</v>
       </c>
-      <c r="T8" s="64"/>
-      <c r="U8" s="64"/>
-      <c r="V8" s="46"/>
-      <c r="W8" s="46"/>
-      <c r="X8" s="46"/>
-      <c r="Y8" s="46"/>
-      <c r="Z8" s="46"/>
-      <c r="AA8" s="46"/>
+      <c r="T8" s="78"/>
+      <c r="U8" s="78"/>
+      <c r="V8" s="79"/>
+      <c r="W8" s="79"/>
+      <c r="X8" s="79"/>
+      <c r="Y8" s="79"/>
+      <c r="Z8" s="79"/>
+      <c r="AA8" s="79"/>
       <c r="AE8" s="6"/>
       <c r="AF8" s="6"/>
       <c r="AG8" s="6"/>
@@ -8743,28 +8739,28 @@
       <c r="AM8" s="6"/>
     </row>
     <row r="9" spans="2:39" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="79"/>
-      <c r="C9" s="79"/>
-      <c r="D9" s="79"/>
-      <c r="E9" s="79"/>
-      <c r="F9" s="79"/>
-      <c r="G9" s="79"/>
-      <c r="H9" s="79"/>
-      <c r="I9" s="79"/>
-      <c r="J9" s="79"/>
-      <c r="K9" s="79"/>
-      <c r="L9" s="79"/>
-      <c r="M9" s="79"/>
-      <c r="N9" s="79"/>
-      <c r="O9" s="79"/>
-      <c r="P9" s="79"/>
-      <c r="Q9" s="79"/>
-      <c r="R9" s="79"/>
-      <c r="S9" s="63" t="s">
+      <c r="B9" s="76"/>
+      <c r="C9" s="76"/>
+      <c r="D9" s="76"/>
+      <c r="E9" s="76"/>
+      <c r="F9" s="76"/>
+      <c r="G9" s="76"/>
+      <c r="H9" s="76"/>
+      <c r="I9" s="76"/>
+      <c r="J9" s="76"/>
+      <c r="K9" s="76"/>
+      <c r="L9" s="76"/>
+      <c r="M9" s="76"/>
+      <c r="N9" s="76"/>
+      <c r="O9" s="76"/>
+      <c r="P9" s="76"/>
+      <c r="Q9" s="76"/>
+      <c r="R9" s="76"/>
+      <c r="S9" s="77" t="s">
         <v>37</v>
       </c>
-      <c r="T9" s="64"/>
-      <c r="U9" s="64"/>
+      <c r="T9" s="78"/>
+      <c r="U9" s="78"/>
       <c r="V9" s="80"/>
       <c r="W9" s="81"/>
       <c r="X9" s="9" t="s">
@@ -8787,995 +8783,995 @@
       <c r="AM9" s="6"/>
     </row>
     <row r="10" spans="2:39" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="108" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="33"/>
-      <c r="D10" s="33"/>
-      <c r="E10" s="42"/>
-      <c r="F10" s="42"/>
-      <c r="G10" s="42"/>
-      <c r="H10" s="42"/>
-      <c r="I10" s="42"/>
-      <c r="J10" s="42"/>
-      <c r="K10" s="33" t="s">
+      <c r="C10" s="108"/>
+      <c r="D10" s="108"/>
+      <c r="E10" s="65"/>
+      <c r="F10" s="65"/>
+      <c r="G10" s="65"/>
+      <c r="H10" s="65"/>
+      <c r="I10" s="65"/>
+      <c r="J10" s="65"/>
+      <c r="K10" s="108" t="s">
         <v>20</v>
       </c>
-      <c r="L10" s="33"/>
-      <c r="M10" s="33"/>
-      <c r="N10" s="36"/>
-      <c r="O10" s="37"/>
-      <c r="P10" s="37"/>
-      <c r="Q10" s="37"/>
-      <c r="R10" s="38"/>
-      <c r="S10" s="33" t="s">
+      <c r="L10" s="108"/>
+      <c r="M10" s="108"/>
+      <c r="N10" s="99"/>
+      <c r="O10" s="100"/>
+      <c r="P10" s="100"/>
+      <c r="Q10" s="100"/>
+      <c r="R10" s="101"/>
+      <c r="S10" s="108" t="s">
         <v>48</v>
       </c>
-      <c r="T10" s="33"/>
-      <c r="U10" s="33"/>
-      <c r="V10" s="43"/>
-      <c r="W10" s="44"/>
-      <c r="X10" s="44"/>
-      <c r="Y10" s="44"/>
-      <c r="Z10" s="44"/>
-      <c r="AA10" s="45"/>
+      <c r="T10" s="108"/>
+      <c r="U10" s="108"/>
+      <c r="V10" s="112"/>
+      <c r="W10" s="113"/>
+      <c r="X10" s="113"/>
+      <c r="Y10" s="113"/>
+      <c r="Z10" s="113"/>
+      <c r="AA10" s="114"/>
     </row>
     <row r="11" spans="2:39" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="108" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="33"/>
-      <c r="D11" s="33"/>
-      <c r="E11" s="42"/>
-      <c r="F11" s="42"/>
-      <c r="G11" s="42"/>
-      <c r="H11" s="42"/>
-      <c r="I11" s="42"/>
-      <c r="J11" s="42"/>
-      <c r="K11" s="33" t="s">
+      <c r="C11" s="108"/>
+      <c r="D11" s="108"/>
+      <c r="E11" s="65"/>
+      <c r="F11" s="65"/>
+      <c r="G11" s="65"/>
+      <c r="H11" s="65"/>
+      <c r="I11" s="65"/>
+      <c r="J11" s="65"/>
+      <c r="K11" s="108" t="s">
         <v>46</v>
       </c>
-      <c r="L11" s="33"/>
-      <c r="M11" s="33"/>
-      <c r="N11" s="36"/>
-      <c r="O11" s="37"/>
-      <c r="P11" s="37"/>
-      <c r="Q11" s="37"/>
-      <c r="R11" s="38"/>
-      <c r="S11" s="33" t="s">
+      <c r="L11" s="108"/>
+      <c r="M11" s="108"/>
+      <c r="N11" s="99"/>
+      <c r="O11" s="100"/>
+      <c r="P11" s="100"/>
+      <c r="Q11" s="100"/>
+      <c r="R11" s="101"/>
+      <c r="S11" s="108" t="s">
         <v>52</v>
       </c>
-      <c r="T11" s="33"/>
-      <c r="U11" s="33"/>
-      <c r="V11" s="46"/>
-      <c r="W11" s="46"/>
-      <c r="X11" s="46"/>
-      <c r="Y11" s="46"/>
-      <c r="Z11" s="46"/>
-      <c r="AA11" s="46"/>
+      <c r="T11" s="108"/>
+      <c r="U11" s="108"/>
+      <c r="V11" s="79"/>
+      <c r="W11" s="79"/>
+      <c r="X11" s="79"/>
+      <c r="Y11" s="79"/>
+      <c r="Z11" s="79"/>
+      <c r="AA11" s="79"/>
     </row>
     <row r="12" spans="2:39" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="108" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="33"/>
-      <c r="D12" s="33"/>
-      <c r="E12" s="42"/>
-      <c r="F12" s="42"/>
-      <c r="G12" s="42"/>
-      <c r="H12" s="42"/>
-      <c r="I12" s="42"/>
-      <c r="J12" s="42"/>
-      <c r="K12" s="33" t="s">
+      <c r="C12" s="108"/>
+      <c r="D12" s="108"/>
+      <c r="E12" s="65"/>
+      <c r="F12" s="65"/>
+      <c r="G12" s="65"/>
+      <c r="H12" s="65"/>
+      <c r="I12" s="65"/>
+      <c r="J12" s="65"/>
+      <c r="K12" s="108" t="s">
         <v>47</v>
       </c>
-      <c r="L12" s="33"/>
-      <c r="M12" s="33"/>
-      <c r="N12" s="36"/>
-      <c r="O12" s="37"/>
-      <c r="P12" s="37"/>
-      <c r="Q12" s="37"/>
-      <c r="R12" s="38"/>
-      <c r="S12" s="33" t="s">
+      <c r="L12" s="108"/>
+      <c r="M12" s="108"/>
+      <c r="N12" s="99"/>
+      <c r="O12" s="100"/>
+      <c r="P12" s="100"/>
+      <c r="Q12" s="100"/>
+      <c r="R12" s="101"/>
+      <c r="S12" s="108" t="s">
         <v>22</v>
       </c>
-      <c r="T12" s="33"/>
-      <c r="U12" s="33"/>
-      <c r="V12" s="47">
+      <c r="T12" s="108"/>
+      <c r="U12" s="108"/>
+      <c r="V12" s="82">
         <f>V8-V11</f>
         <v>0</v>
       </c>
-      <c r="W12" s="47"/>
-      <c r="X12" s="47"/>
-      <c r="Y12" s="47"/>
-      <c r="Z12" s="47"/>
-      <c r="AA12" s="47"/>
+      <c r="W12" s="82"/>
+      <c r="X12" s="82"/>
+      <c r="Y12" s="82"/>
+      <c r="Z12" s="82"/>
+      <c r="AA12" s="82"/>
     </row>
     <row r="13" spans="2:39" ht="6.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="35"/>
-      <c r="H13" s="35"/>
-      <c r="I13" s="35"/>
-      <c r="J13" s="35"/>
-      <c r="K13" s="35"/>
-      <c r="L13" s="35"/>
-      <c r="M13" s="35"/>
-      <c r="N13" s="35"/>
-      <c r="O13" s="35"/>
-      <c r="P13" s="35"/>
-      <c r="Q13" s="35"/>
-      <c r="R13" s="35"/>
-      <c r="S13" s="35"/>
-      <c r="T13" s="35"/>
-      <c r="U13" s="35"/>
-      <c r="V13" s="35"/>
-      <c r="W13" s="35"/>
-      <c r="X13" s="35"/>
-      <c r="Y13" s="35"/>
-      <c r="Z13" s="35"/>
-      <c r="AA13" s="35"/>
+      <c r="B13" s="31"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="31"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="31"/>
+      <c r="I13" s="31"/>
+      <c r="J13" s="31"/>
+      <c r="K13" s="31"/>
+      <c r="L13" s="31"/>
+      <c r="M13" s="31"/>
+      <c r="N13" s="31"/>
+      <c r="O13" s="31"/>
+      <c r="P13" s="31"/>
+      <c r="Q13" s="31"/>
+      <c r="R13" s="31"/>
+      <c r="S13" s="31"/>
+      <c r="T13" s="31"/>
+      <c r="U13" s="31"/>
+      <c r="V13" s="31"/>
+      <c r="W13" s="31"/>
+      <c r="X13" s="31"/>
+      <c r="Y13" s="31"/>
+      <c r="Z13" s="31"/>
+      <c r="AA13" s="31"/>
     </row>
     <row r="14" spans="2:39" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="109" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="26"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="26"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="26"/>
-      <c r="J14" s="26"/>
-      <c r="K14" s="26"/>
-      <c r="L14" s="26"/>
-      <c r="M14" s="26"/>
-      <c r="N14" s="26"/>
-      <c r="O14" s="26"/>
-      <c r="P14" s="26"/>
-      <c r="Q14" s="27"/>
-      <c r="R14" s="63" t="s">
+      <c r="C14" s="110"/>
+      <c r="D14" s="110"/>
+      <c r="E14" s="110"/>
+      <c r="F14" s="110"/>
+      <c r="G14" s="110"/>
+      <c r="H14" s="110"/>
+      <c r="I14" s="110"/>
+      <c r="J14" s="110"/>
+      <c r="K14" s="110"/>
+      <c r="L14" s="110"/>
+      <c r="M14" s="110"/>
+      <c r="N14" s="110"/>
+      <c r="O14" s="110"/>
+      <c r="P14" s="110"/>
+      <c r="Q14" s="111"/>
+      <c r="R14" s="77" t="s">
         <v>40</v>
       </c>
-      <c r="S14" s="64"/>
-      <c r="T14" s="64"/>
-      <c r="U14" s="64"/>
-      <c r="V14" s="65"/>
-      <c r="W14" s="63" t="s">
+      <c r="S14" s="78"/>
+      <c r="T14" s="78"/>
+      <c r="U14" s="78"/>
+      <c r="V14" s="62"/>
+      <c r="W14" s="77" t="s">
         <v>41</v>
       </c>
-      <c r="X14" s="64"/>
-      <c r="Y14" s="64"/>
-      <c r="Z14" s="64"/>
-      <c r="AA14" s="65"/>
+      <c r="X14" s="78"/>
+      <c r="Y14" s="78"/>
+      <c r="Z14" s="78"/>
+      <c r="AA14" s="62"/>
     </row>
     <row r="15" spans="2:39" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="39"/>
-      <c r="C15" s="40"/>
-      <c r="D15" s="40"/>
-      <c r="E15" s="40"/>
-      <c r="F15" s="40"/>
-      <c r="G15" s="40"/>
-      <c r="H15" s="40"/>
-      <c r="I15" s="40"/>
-      <c r="J15" s="40"/>
-      <c r="K15" s="40"/>
-      <c r="L15" s="40"/>
-      <c r="M15" s="40"/>
-      <c r="N15" s="40"/>
-      <c r="O15" s="40"/>
-      <c r="P15" s="40"/>
-      <c r="Q15" s="41"/>
-      <c r="R15" s="53"/>
-      <c r="S15" s="54"/>
-      <c r="T15" s="54"/>
-      <c r="U15" s="54"/>
-      <c r="V15" s="54"/>
-      <c r="W15" s="53"/>
-      <c r="X15" s="54"/>
-      <c r="Y15" s="54"/>
-      <c r="Z15" s="54"/>
-      <c r="AA15" s="59"/>
+      <c r="B15" s="102"/>
+      <c r="C15" s="103"/>
+      <c r="D15" s="103"/>
+      <c r="E15" s="103"/>
+      <c r="F15" s="103"/>
+      <c r="G15" s="103"/>
+      <c r="H15" s="103"/>
+      <c r="I15" s="103"/>
+      <c r="J15" s="103"/>
+      <c r="K15" s="103"/>
+      <c r="L15" s="103"/>
+      <c r="M15" s="103"/>
+      <c r="N15" s="103"/>
+      <c r="O15" s="103"/>
+      <c r="P15" s="103"/>
+      <c r="Q15" s="104"/>
+      <c r="R15" s="88"/>
+      <c r="S15" s="89"/>
+      <c r="T15" s="89"/>
+      <c r="U15" s="89"/>
+      <c r="V15" s="89"/>
+      <c r="W15" s="88"/>
+      <c r="X15" s="89"/>
+      <c r="Y15" s="89"/>
+      <c r="Z15" s="89"/>
+      <c r="AA15" s="94"/>
     </row>
     <row r="16" spans="2:39" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="109" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
-      <c r="H16" s="26"/>
-      <c r="I16" s="26"/>
-      <c r="J16" s="26"/>
-      <c r="K16" s="26"/>
-      <c r="L16" s="26"/>
-      <c r="M16" s="26"/>
-      <c r="N16" s="26"/>
-      <c r="O16" s="26"/>
-      <c r="P16" s="26"/>
-      <c r="Q16" s="27"/>
-      <c r="R16" s="55"/>
-      <c r="S16" s="56"/>
-      <c r="T16" s="56"/>
-      <c r="U16" s="56"/>
-      <c r="V16" s="56"/>
-      <c r="W16" s="55"/>
-      <c r="X16" s="56"/>
-      <c r="Y16" s="56"/>
-      <c r="Z16" s="56"/>
-      <c r="AA16" s="60"/>
+      <c r="C16" s="110"/>
+      <c r="D16" s="110"/>
+      <c r="E16" s="110"/>
+      <c r="F16" s="110"/>
+      <c r="G16" s="110"/>
+      <c r="H16" s="110"/>
+      <c r="I16" s="110"/>
+      <c r="J16" s="110"/>
+      <c r="K16" s="110"/>
+      <c r="L16" s="110"/>
+      <c r="M16" s="110"/>
+      <c r="N16" s="110"/>
+      <c r="O16" s="110"/>
+      <c r="P16" s="110"/>
+      <c r="Q16" s="111"/>
+      <c r="R16" s="90"/>
+      <c r="S16" s="91"/>
+      <c r="T16" s="91"/>
+      <c r="U16" s="91"/>
+      <c r="V16" s="91"/>
+      <c r="W16" s="90"/>
+      <c r="X16" s="91"/>
+      <c r="Y16" s="91"/>
+      <c r="Z16" s="91"/>
+      <c r="AA16" s="95"/>
     </row>
     <row r="17" spans="2:27" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="39"/>
-      <c r="C17" s="40"/>
-      <c r="D17" s="40"/>
-      <c r="E17" s="40"/>
-      <c r="F17" s="40"/>
-      <c r="G17" s="40"/>
-      <c r="H17" s="40"/>
-      <c r="I17" s="40"/>
-      <c r="J17" s="40"/>
-      <c r="K17" s="40"/>
-      <c r="L17" s="40"/>
-      <c r="M17" s="40"/>
-      <c r="N17" s="40"/>
-      <c r="O17" s="40"/>
-      <c r="P17" s="40"/>
-      <c r="Q17" s="41"/>
-      <c r="R17" s="55"/>
-      <c r="S17" s="56"/>
-      <c r="T17" s="56"/>
-      <c r="U17" s="56"/>
-      <c r="V17" s="56"/>
-      <c r="W17" s="55"/>
-      <c r="X17" s="56"/>
-      <c r="Y17" s="56"/>
-      <c r="Z17" s="56"/>
-      <c r="AA17" s="60"/>
+      <c r="B17" s="102"/>
+      <c r="C17" s="103"/>
+      <c r="D17" s="103"/>
+      <c r="E17" s="103"/>
+      <c r="F17" s="103"/>
+      <c r="G17" s="103"/>
+      <c r="H17" s="103"/>
+      <c r="I17" s="103"/>
+      <c r="J17" s="103"/>
+      <c r="K17" s="103"/>
+      <c r="L17" s="103"/>
+      <c r="M17" s="103"/>
+      <c r="N17" s="103"/>
+      <c r="O17" s="103"/>
+      <c r="P17" s="103"/>
+      <c r="Q17" s="104"/>
+      <c r="R17" s="90"/>
+      <c r="S17" s="91"/>
+      <c r="T17" s="91"/>
+      <c r="U17" s="91"/>
+      <c r="V17" s="91"/>
+      <c r="W17" s="90"/>
+      <c r="X17" s="91"/>
+      <c r="Y17" s="91"/>
+      <c r="Z17" s="91"/>
+      <c r="AA17" s="95"/>
     </row>
     <row r="18" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="25" t="s">
+      <c r="B18" s="109" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="26"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="26"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="26"/>
-      <c r="J18" s="26"/>
-      <c r="K18" s="26"/>
-      <c r="L18" s="26"/>
-      <c r="M18" s="26"/>
-      <c r="N18" s="26"/>
-      <c r="O18" s="26"/>
-      <c r="P18" s="26"/>
-      <c r="Q18" s="27"/>
-      <c r="R18" s="55"/>
-      <c r="S18" s="56"/>
-      <c r="T18" s="56"/>
-      <c r="U18" s="56"/>
-      <c r="V18" s="56"/>
-      <c r="W18" s="55"/>
-      <c r="X18" s="56"/>
-      <c r="Y18" s="56"/>
-      <c r="Z18" s="56"/>
-      <c r="AA18" s="60"/>
+      <c r="C18" s="110"/>
+      <c r="D18" s="110"/>
+      <c r="E18" s="110"/>
+      <c r="F18" s="110"/>
+      <c r="G18" s="110"/>
+      <c r="H18" s="110"/>
+      <c r="I18" s="110"/>
+      <c r="J18" s="110"/>
+      <c r="K18" s="110"/>
+      <c r="L18" s="110"/>
+      <c r="M18" s="110"/>
+      <c r="N18" s="110"/>
+      <c r="O18" s="110"/>
+      <c r="P18" s="110"/>
+      <c r="Q18" s="111"/>
+      <c r="R18" s="90"/>
+      <c r="S18" s="91"/>
+      <c r="T18" s="91"/>
+      <c r="U18" s="91"/>
+      <c r="V18" s="91"/>
+      <c r="W18" s="90"/>
+      <c r="X18" s="91"/>
+      <c r="Y18" s="91"/>
+      <c r="Z18" s="91"/>
+      <c r="AA18" s="95"/>
     </row>
     <row r="19" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="39"/>
-      <c r="C19" s="40"/>
-      <c r="D19" s="40"/>
-      <c r="E19" s="40"/>
-      <c r="F19" s="40"/>
-      <c r="G19" s="40"/>
-      <c r="H19" s="40"/>
-      <c r="I19" s="40"/>
-      <c r="J19" s="40"/>
-      <c r="K19" s="40"/>
-      <c r="L19" s="40"/>
-      <c r="M19" s="40"/>
-      <c r="N19" s="40"/>
-      <c r="O19" s="40"/>
-      <c r="P19" s="40"/>
-      <c r="Q19" s="41"/>
-      <c r="R19" s="55"/>
-      <c r="S19" s="56"/>
-      <c r="T19" s="56"/>
-      <c r="U19" s="56"/>
-      <c r="V19" s="56"/>
-      <c r="W19" s="55"/>
-      <c r="X19" s="56"/>
-      <c r="Y19" s="56"/>
-      <c r="Z19" s="56"/>
-      <c r="AA19" s="60"/>
+      <c r="B19" s="102"/>
+      <c r="C19" s="103"/>
+      <c r="D19" s="103"/>
+      <c r="E19" s="103"/>
+      <c r="F19" s="103"/>
+      <c r="G19" s="103"/>
+      <c r="H19" s="103"/>
+      <c r="I19" s="103"/>
+      <c r="J19" s="103"/>
+      <c r="K19" s="103"/>
+      <c r="L19" s="103"/>
+      <c r="M19" s="103"/>
+      <c r="N19" s="103"/>
+      <c r="O19" s="103"/>
+      <c r="P19" s="103"/>
+      <c r="Q19" s="104"/>
+      <c r="R19" s="90"/>
+      <c r="S19" s="91"/>
+      <c r="T19" s="91"/>
+      <c r="U19" s="91"/>
+      <c r="V19" s="91"/>
+      <c r="W19" s="90"/>
+      <c r="X19" s="91"/>
+      <c r="Y19" s="91"/>
+      <c r="Z19" s="91"/>
+      <c r="AA19" s="95"/>
     </row>
     <row r="20" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="66"/>
-      <c r="C20" s="67"/>
-      <c r="D20" s="67"/>
-      <c r="E20" s="67"/>
-      <c r="F20" s="67"/>
-      <c r="G20" s="67"/>
-      <c r="H20" s="67"/>
-      <c r="I20" s="67"/>
-      <c r="J20" s="67"/>
-      <c r="K20" s="67"/>
-      <c r="L20" s="67"/>
-      <c r="M20" s="67"/>
-      <c r="N20" s="67"/>
-      <c r="O20" s="67"/>
-      <c r="P20" s="67"/>
-      <c r="Q20" s="68"/>
-      <c r="R20" s="55"/>
-      <c r="S20" s="56"/>
-      <c r="T20" s="56"/>
-      <c r="U20" s="56"/>
-      <c r="V20" s="56"/>
-      <c r="W20" s="55"/>
-      <c r="X20" s="56"/>
-      <c r="Y20" s="56"/>
-      <c r="Z20" s="56"/>
-      <c r="AA20" s="60"/>
+      <c r="B20" s="105"/>
+      <c r="C20" s="106"/>
+      <c r="D20" s="106"/>
+      <c r="E20" s="106"/>
+      <c r="F20" s="106"/>
+      <c r="G20" s="106"/>
+      <c r="H20" s="106"/>
+      <c r="I20" s="106"/>
+      <c r="J20" s="106"/>
+      <c r="K20" s="106"/>
+      <c r="L20" s="106"/>
+      <c r="M20" s="106"/>
+      <c r="N20" s="106"/>
+      <c r="O20" s="106"/>
+      <c r="P20" s="106"/>
+      <c r="Q20" s="107"/>
+      <c r="R20" s="90"/>
+      <c r="S20" s="91"/>
+      <c r="T20" s="91"/>
+      <c r="U20" s="91"/>
+      <c r="V20" s="91"/>
+      <c r="W20" s="90"/>
+      <c r="X20" s="91"/>
+      <c r="Y20" s="91"/>
+      <c r="Z20" s="91"/>
+      <c r="AA20" s="95"/>
     </row>
     <row r="21" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="48" t="s">
+      <c r="B21" s="83" t="s">
         <v>0</v>
       </c>
-      <c r="C21" s="49"/>
-      <c r="D21" s="49"/>
-      <c r="E21" s="49"/>
-      <c r="F21" s="49"/>
-      <c r="G21" s="49"/>
-      <c r="H21" s="49"/>
-      <c r="I21" s="49"/>
-      <c r="J21" s="49"/>
-      <c r="K21" s="49"/>
-      <c r="L21" s="49"/>
-      <c r="M21" s="49"/>
-      <c r="N21" s="49"/>
-      <c r="O21" s="49"/>
-      <c r="P21" s="49"/>
-      <c r="Q21" s="50"/>
-      <c r="R21" s="57"/>
-      <c r="S21" s="58"/>
-      <c r="T21" s="58"/>
-      <c r="U21" s="58"/>
-      <c r="V21" s="58"/>
-      <c r="W21" s="57"/>
-      <c r="X21" s="58"/>
-      <c r="Y21" s="58"/>
-      <c r="Z21" s="58"/>
-      <c r="AA21" s="61"/>
+      <c r="C21" s="84"/>
+      <c r="D21" s="84"/>
+      <c r="E21" s="84"/>
+      <c r="F21" s="84"/>
+      <c r="G21" s="84"/>
+      <c r="H21" s="84"/>
+      <c r="I21" s="84"/>
+      <c r="J21" s="84"/>
+      <c r="K21" s="84"/>
+      <c r="L21" s="84"/>
+      <c r="M21" s="84"/>
+      <c r="N21" s="84"/>
+      <c r="O21" s="84"/>
+      <c r="P21" s="84"/>
+      <c r="Q21" s="85"/>
+      <c r="R21" s="92"/>
+      <c r="S21" s="93"/>
+      <c r="T21" s="93"/>
+      <c r="U21" s="93"/>
+      <c r="V21" s="93"/>
+      <c r="W21" s="92"/>
+      <c r="X21" s="93"/>
+      <c r="Y21" s="93"/>
+      <c r="Z21" s="93"/>
+      <c r="AA21" s="96"/>
     </row>
     <row r="22" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="51"/>
-      <c r="C22" s="52"/>
-      <c r="D22" s="52"/>
-      <c r="E22" s="52"/>
-      <c r="F22" s="52"/>
-      <c r="G22" s="52"/>
-      <c r="H22" s="52"/>
-      <c r="I22" s="52"/>
-      <c r="J22" s="52"/>
-      <c r="K22" s="52"/>
-      <c r="L22" s="52"/>
-      <c r="M22" s="52"/>
-      <c r="N22" s="52"/>
-      <c r="O22" s="52"/>
-      <c r="P22" s="52"/>
-      <c r="Q22" s="52"/>
-      <c r="R22" s="62"/>
-      <c r="S22" s="34"/>
-      <c r="T22" s="34"/>
-      <c r="U22" s="34"/>
-      <c r="V22" s="34"/>
-      <c r="W22" s="34"/>
-      <c r="X22" s="34"/>
-      <c r="Y22" s="34"/>
-      <c r="Z22" s="34"/>
-      <c r="AA22" s="34"/>
+      <c r="B22" s="86"/>
+      <c r="C22" s="87"/>
+      <c r="D22" s="87"/>
+      <c r="E22" s="87"/>
+      <c r="F22" s="87"/>
+      <c r="G22" s="87"/>
+      <c r="H22" s="87"/>
+      <c r="I22" s="87"/>
+      <c r="J22" s="87"/>
+      <c r="K22" s="87"/>
+      <c r="L22" s="87"/>
+      <c r="M22" s="87"/>
+      <c r="N22" s="87"/>
+      <c r="O22" s="87"/>
+      <c r="P22" s="87"/>
+      <c r="Q22" s="87"/>
+      <c r="R22" s="97"/>
+      <c r="S22" s="98"/>
+      <c r="T22" s="98"/>
+      <c r="U22" s="98"/>
+      <c r="V22" s="98"/>
+      <c r="W22" s="98"/>
+      <c r="X22" s="98"/>
+      <c r="Y22" s="98"/>
+      <c r="Z22" s="98"/>
+      <c r="AA22" s="98"/>
     </row>
     <row r="23" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="52"/>
-      <c r="C23" s="52"/>
-      <c r="D23" s="52"/>
-      <c r="E23" s="52"/>
-      <c r="F23" s="52"/>
-      <c r="G23" s="52"/>
-      <c r="H23" s="52"/>
-      <c r="I23" s="52"/>
-      <c r="J23" s="52"/>
-      <c r="K23" s="52"/>
-      <c r="L23" s="52"/>
-      <c r="M23" s="52"/>
-      <c r="N23" s="52"/>
-      <c r="O23" s="52"/>
-      <c r="P23" s="52"/>
-      <c r="Q23" s="52"/>
-      <c r="R23" s="34"/>
-      <c r="S23" s="34"/>
-      <c r="T23" s="34"/>
-      <c r="U23" s="34"/>
-      <c r="V23" s="34"/>
-      <c r="W23" s="34"/>
-      <c r="X23" s="34"/>
-      <c r="Y23" s="34"/>
-      <c r="Z23" s="34"/>
-      <c r="AA23" s="34"/>
+      <c r="B23" s="87"/>
+      <c r="C23" s="87"/>
+      <c r="D23" s="87"/>
+      <c r="E23" s="87"/>
+      <c r="F23" s="87"/>
+      <c r="G23" s="87"/>
+      <c r="H23" s="87"/>
+      <c r="I23" s="87"/>
+      <c r="J23" s="87"/>
+      <c r="K23" s="87"/>
+      <c r="L23" s="87"/>
+      <c r="M23" s="87"/>
+      <c r="N23" s="87"/>
+      <c r="O23" s="87"/>
+      <c r="P23" s="87"/>
+      <c r="Q23" s="87"/>
+      <c r="R23" s="98"/>
+      <c r="S23" s="98"/>
+      <c r="T23" s="98"/>
+      <c r="U23" s="98"/>
+      <c r="V23" s="98"/>
+      <c r="W23" s="98"/>
+      <c r="X23" s="98"/>
+      <c r="Y23" s="98"/>
+      <c r="Z23" s="98"/>
+      <c r="AA23" s="98"/>
     </row>
     <row r="24" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="52"/>
-      <c r="C24" s="52"/>
-      <c r="D24" s="52"/>
-      <c r="E24" s="52"/>
-      <c r="F24" s="52"/>
-      <c r="G24" s="52"/>
-      <c r="H24" s="52"/>
-      <c r="I24" s="52"/>
-      <c r="J24" s="52"/>
-      <c r="K24" s="52"/>
-      <c r="L24" s="52"/>
-      <c r="M24" s="52"/>
-      <c r="N24" s="52"/>
-      <c r="O24" s="52"/>
-      <c r="P24" s="52"/>
-      <c r="Q24" s="52"/>
-      <c r="R24" s="34"/>
-      <c r="S24" s="34"/>
-      <c r="T24" s="34"/>
-      <c r="U24" s="34"/>
-      <c r="V24" s="34"/>
-      <c r="W24" s="34"/>
-      <c r="X24" s="34"/>
-      <c r="Y24" s="34"/>
-      <c r="Z24" s="34"/>
-      <c r="AA24" s="34"/>
+      <c r="B24" s="87"/>
+      <c r="C24" s="87"/>
+      <c r="D24" s="87"/>
+      <c r="E24" s="87"/>
+      <c r="F24" s="87"/>
+      <c r="G24" s="87"/>
+      <c r="H24" s="87"/>
+      <c r="I24" s="87"/>
+      <c r="J24" s="87"/>
+      <c r="K24" s="87"/>
+      <c r="L24" s="87"/>
+      <c r="M24" s="87"/>
+      <c r="N24" s="87"/>
+      <c r="O24" s="87"/>
+      <c r="P24" s="87"/>
+      <c r="Q24" s="87"/>
+      <c r="R24" s="98"/>
+      <c r="S24" s="98"/>
+      <c r="T24" s="98"/>
+      <c r="U24" s="98"/>
+      <c r="V24" s="98"/>
+      <c r="W24" s="98"/>
+      <c r="X24" s="98"/>
+      <c r="Y24" s="98"/>
+      <c r="Z24" s="98"/>
+      <c r="AA24" s="98"/>
     </row>
     <row r="25" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="52"/>
-      <c r="C25" s="52"/>
-      <c r="D25" s="52"/>
-      <c r="E25" s="52"/>
-      <c r="F25" s="52"/>
-      <c r="G25" s="52"/>
-      <c r="H25" s="52"/>
-      <c r="I25" s="52"/>
-      <c r="J25" s="52"/>
-      <c r="K25" s="52"/>
-      <c r="L25" s="52"/>
-      <c r="M25" s="52"/>
-      <c r="N25" s="52"/>
-      <c r="O25" s="52"/>
-      <c r="P25" s="52"/>
-      <c r="Q25" s="52"/>
-      <c r="R25" s="34"/>
-      <c r="S25" s="34"/>
-      <c r="T25" s="34"/>
-      <c r="U25" s="34"/>
-      <c r="V25" s="34"/>
-      <c r="W25" s="34"/>
-      <c r="X25" s="34"/>
-      <c r="Y25" s="34"/>
-      <c r="Z25" s="34"/>
-      <c r="AA25" s="34"/>
+      <c r="B25" s="87"/>
+      <c r="C25" s="87"/>
+      <c r="D25" s="87"/>
+      <c r="E25" s="87"/>
+      <c r="F25" s="87"/>
+      <c r="G25" s="87"/>
+      <c r="H25" s="87"/>
+      <c r="I25" s="87"/>
+      <c r="J25" s="87"/>
+      <c r="K25" s="87"/>
+      <c r="L25" s="87"/>
+      <c r="M25" s="87"/>
+      <c r="N25" s="87"/>
+      <c r="O25" s="87"/>
+      <c r="P25" s="87"/>
+      <c r="Q25" s="87"/>
+      <c r="R25" s="98"/>
+      <c r="S25" s="98"/>
+      <c r="T25" s="98"/>
+      <c r="U25" s="98"/>
+      <c r="V25" s="98"/>
+      <c r="W25" s="98"/>
+      <c r="X25" s="98"/>
+      <c r="Y25" s="98"/>
+      <c r="Z25" s="98"/>
+      <c r="AA25" s="98"/>
     </row>
     <row r="26" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="52"/>
-      <c r="C26" s="52"/>
-      <c r="D26" s="52"/>
-      <c r="E26" s="52"/>
-      <c r="F26" s="52"/>
-      <c r="G26" s="52"/>
-      <c r="H26" s="52"/>
-      <c r="I26" s="52"/>
-      <c r="J26" s="52"/>
-      <c r="K26" s="52"/>
-      <c r="L26" s="52"/>
-      <c r="M26" s="52"/>
-      <c r="N26" s="52"/>
-      <c r="O26" s="52"/>
-      <c r="P26" s="52"/>
-      <c r="Q26" s="52"/>
-      <c r="R26" s="34"/>
-      <c r="S26" s="34"/>
-      <c r="T26" s="34"/>
-      <c r="U26" s="34"/>
-      <c r="V26" s="34"/>
-      <c r="W26" s="34"/>
-      <c r="X26" s="34"/>
-      <c r="Y26" s="34"/>
-      <c r="Z26" s="34"/>
-      <c r="AA26" s="34"/>
+      <c r="B26" s="87"/>
+      <c r="C26" s="87"/>
+      <c r="D26" s="87"/>
+      <c r="E26" s="87"/>
+      <c r="F26" s="87"/>
+      <c r="G26" s="87"/>
+      <c r="H26" s="87"/>
+      <c r="I26" s="87"/>
+      <c r="J26" s="87"/>
+      <c r="K26" s="87"/>
+      <c r="L26" s="87"/>
+      <c r="M26" s="87"/>
+      <c r="N26" s="87"/>
+      <c r="O26" s="87"/>
+      <c r="P26" s="87"/>
+      <c r="Q26" s="87"/>
+      <c r="R26" s="98"/>
+      <c r="S26" s="98"/>
+      <c r="T26" s="98"/>
+      <c r="U26" s="98"/>
+      <c r="V26" s="98"/>
+      <c r="W26" s="98"/>
+      <c r="X26" s="98"/>
+      <c r="Y26" s="98"/>
+      <c r="Z26" s="98"/>
+      <c r="AA26" s="98"/>
     </row>
     <row r="27" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="52"/>
-      <c r="C27" s="52"/>
-      <c r="D27" s="52"/>
-      <c r="E27" s="52"/>
-      <c r="F27" s="52"/>
-      <c r="G27" s="52"/>
-      <c r="H27" s="52"/>
-      <c r="I27" s="52"/>
-      <c r="J27" s="52"/>
-      <c r="K27" s="52"/>
-      <c r="L27" s="52"/>
-      <c r="M27" s="52"/>
-      <c r="N27" s="52"/>
-      <c r="O27" s="52"/>
-      <c r="P27" s="52"/>
-      <c r="Q27" s="52"/>
-      <c r="R27" s="34"/>
-      <c r="S27" s="34"/>
-      <c r="T27" s="34"/>
-      <c r="U27" s="34"/>
-      <c r="V27" s="34"/>
-      <c r="W27" s="34"/>
-      <c r="X27" s="34"/>
-      <c r="Y27" s="34"/>
-      <c r="Z27" s="34"/>
-      <c r="AA27" s="34"/>
+      <c r="B27" s="87"/>
+      <c r="C27" s="87"/>
+      <c r="D27" s="87"/>
+      <c r="E27" s="87"/>
+      <c r="F27" s="87"/>
+      <c r="G27" s="87"/>
+      <c r="H27" s="87"/>
+      <c r="I27" s="87"/>
+      <c r="J27" s="87"/>
+      <c r="K27" s="87"/>
+      <c r="L27" s="87"/>
+      <c r="M27" s="87"/>
+      <c r="N27" s="87"/>
+      <c r="O27" s="87"/>
+      <c r="P27" s="87"/>
+      <c r="Q27" s="87"/>
+      <c r="R27" s="98"/>
+      <c r="S27" s="98"/>
+      <c r="T27" s="98"/>
+      <c r="U27" s="98"/>
+      <c r="V27" s="98"/>
+      <c r="W27" s="98"/>
+      <c r="X27" s="98"/>
+      <c r="Y27" s="98"/>
+      <c r="Z27" s="98"/>
+      <c r="AA27" s="98"/>
     </row>
     <row r="28" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="52"/>
-      <c r="C28" s="52"/>
-      <c r="D28" s="52"/>
-      <c r="E28" s="52"/>
-      <c r="F28" s="52"/>
-      <c r="G28" s="52"/>
-      <c r="H28" s="52"/>
-      <c r="I28" s="52"/>
-      <c r="J28" s="52"/>
-      <c r="K28" s="52"/>
-      <c r="L28" s="52"/>
-      <c r="M28" s="52"/>
-      <c r="N28" s="52"/>
-      <c r="O28" s="52"/>
-      <c r="P28" s="52"/>
-      <c r="Q28" s="52"/>
-      <c r="R28" s="62"/>
-      <c r="S28" s="34"/>
-      <c r="T28" s="34"/>
-      <c r="U28" s="34"/>
-      <c r="V28" s="34"/>
-      <c r="W28" s="34"/>
-      <c r="X28" s="34"/>
-      <c r="Y28" s="34"/>
-      <c r="Z28" s="34"/>
-      <c r="AA28" s="34"/>
+      <c r="B28" s="87"/>
+      <c r="C28" s="87"/>
+      <c r="D28" s="87"/>
+      <c r="E28" s="87"/>
+      <c r="F28" s="87"/>
+      <c r="G28" s="87"/>
+      <c r="H28" s="87"/>
+      <c r="I28" s="87"/>
+      <c r="J28" s="87"/>
+      <c r="K28" s="87"/>
+      <c r="L28" s="87"/>
+      <c r="M28" s="87"/>
+      <c r="N28" s="87"/>
+      <c r="O28" s="87"/>
+      <c r="P28" s="87"/>
+      <c r="Q28" s="87"/>
+      <c r="R28" s="97"/>
+      <c r="S28" s="98"/>
+      <c r="T28" s="98"/>
+      <c r="U28" s="98"/>
+      <c r="V28" s="98"/>
+      <c r="W28" s="98"/>
+      <c r="X28" s="98"/>
+      <c r="Y28" s="98"/>
+      <c r="Z28" s="98"/>
+      <c r="AA28" s="98"/>
     </row>
     <row r="29" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="52"/>
-      <c r="C29" s="52"/>
-      <c r="D29" s="52"/>
-      <c r="E29" s="52"/>
-      <c r="F29" s="52"/>
-      <c r="G29" s="52"/>
-      <c r="H29" s="52"/>
-      <c r="I29" s="52"/>
-      <c r="J29" s="52"/>
-      <c r="K29" s="52"/>
-      <c r="L29" s="52"/>
-      <c r="M29" s="52"/>
-      <c r="N29" s="52"/>
-      <c r="O29" s="52"/>
-      <c r="P29" s="52"/>
-      <c r="Q29" s="52"/>
-      <c r="R29" s="34"/>
-      <c r="S29" s="34"/>
-      <c r="T29" s="34"/>
-      <c r="U29" s="34"/>
-      <c r="V29" s="34"/>
-      <c r="W29" s="34"/>
-      <c r="X29" s="34"/>
-      <c r="Y29" s="34"/>
-      <c r="Z29" s="34"/>
-      <c r="AA29" s="34"/>
+      <c r="B29" s="87"/>
+      <c r="C29" s="87"/>
+      <c r="D29" s="87"/>
+      <c r="E29" s="87"/>
+      <c r="F29" s="87"/>
+      <c r="G29" s="87"/>
+      <c r="H29" s="87"/>
+      <c r="I29" s="87"/>
+      <c r="J29" s="87"/>
+      <c r="K29" s="87"/>
+      <c r="L29" s="87"/>
+      <c r="M29" s="87"/>
+      <c r="N29" s="87"/>
+      <c r="O29" s="87"/>
+      <c r="P29" s="87"/>
+      <c r="Q29" s="87"/>
+      <c r="R29" s="98"/>
+      <c r="S29" s="98"/>
+      <c r="T29" s="98"/>
+      <c r="U29" s="98"/>
+      <c r="V29" s="98"/>
+      <c r="W29" s="98"/>
+      <c r="X29" s="98"/>
+      <c r="Y29" s="98"/>
+      <c r="Z29" s="98"/>
+      <c r="AA29" s="98"/>
     </row>
     <row r="30" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="52"/>
-      <c r="C30" s="52"/>
-      <c r="D30" s="52"/>
-      <c r="E30" s="52"/>
-      <c r="F30" s="52"/>
-      <c r="G30" s="52"/>
-      <c r="H30" s="52"/>
-      <c r="I30" s="52"/>
-      <c r="J30" s="52"/>
-      <c r="K30" s="52"/>
-      <c r="L30" s="52"/>
-      <c r="M30" s="52"/>
-      <c r="N30" s="52"/>
-      <c r="O30" s="52"/>
-      <c r="P30" s="52"/>
-      <c r="Q30" s="52"/>
-      <c r="R30" s="34"/>
-      <c r="S30" s="34"/>
-      <c r="T30" s="34"/>
-      <c r="U30" s="34"/>
-      <c r="V30" s="34"/>
-      <c r="W30" s="34"/>
-      <c r="X30" s="34"/>
-      <c r="Y30" s="34"/>
-      <c r="Z30" s="34"/>
-      <c r="AA30" s="34"/>
+      <c r="B30" s="87"/>
+      <c r="C30" s="87"/>
+      <c r="D30" s="87"/>
+      <c r="E30" s="87"/>
+      <c r="F30" s="87"/>
+      <c r="G30" s="87"/>
+      <c r="H30" s="87"/>
+      <c r="I30" s="87"/>
+      <c r="J30" s="87"/>
+      <c r="K30" s="87"/>
+      <c r="L30" s="87"/>
+      <c r="M30" s="87"/>
+      <c r="N30" s="87"/>
+      <c r="O30" s="87"/>
+      <c r="P30" s="87"/>
+      <c r="Q30" s="87"/>
+      <c r="R30" s="98"/>
+      <c r="S30" s="98"/>
+      <c r="T30" s="98"/>
+      <c r="U30" s="98"/>
+      <c r="V30" s="98"/>
+      <c r="W30" s="98"/>
+      <c r="X30" s="98"/>
+      <c r="Y30" s="98"/>
+      <c r="Z30" s="98"/>
+      <c r="AA30" s="98"/>
     </row>
     <row r="31" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="52"/>
-      <c r="C31" s="52"/>
-      <c r="D31" s="52"/>
-      <c r="E31" s="52"/>
-      <c r="F31" s="52"/>
-      <c r="G31" s="52"/>
-      <c r="H31" s="52"/>
-      <c r="I31" s="52"/>
-      <c r="J31" s="52"/>
-      <c r="K31" s="52"/>
-      <c r="L31" s="52"/>
-      <c r="M31" s="52"/>
-      <c r="N31" s="52"/>
-      <c r="O31" s="52"/>
-      <c r="P31" s="52"/>
-      <c r="Q31" s="52"/>
-      <c r="R31" s="34"/>
-      <c r="S31" s="34"/>
-      <c r="T31" s="34"/>
-      <c r="U31" s="34"/>
-      <c r="V31" s="34"/>
-      <c r="W31" s="34"/>
-      <c r="X31" s="34"/>
-      <c r="Y31" s="34"/>
-      <c r="Z31" s="34"/>
-      <c r="AA31" s="34"/>
+      <c r="B31" s="87"/>
+      <c r="C31" s="87"/>
+      <c r="D31" s="87"/>
+      <c r="E31" s="87"/>
+      <c r="F31" s="87"/>
+      <c r="G31" s="87"/>
+      <c r="H31" s="87"/>
+      <c r="I31" s="87"/>
+      <c r="J31" s="87"/>
+      <c r="K31" s="87"/>
+      <c r="L31" s="87"/>
+      <c r="M31" s="87"/>
+      <c r="N31" s="87"/>
+      <c r="O31" s="87"/>
+      <c r="P31" s="87"/>
+      <c r="Q31" s="87"/>
+      <c r="R31" s="98"/>
+      <c r="S31" s="98"/>
+      <c r="T31" s="98"/>
+      <c r="U31" s="98"/>
+      <c r="V31" s="98"/>
+      <c r="W31" s="98"/>
+      <c r="X31" s="98"/>
+      <c r="Y31" s="98"/>
+      <c r="Z31" s="98"/>
+      <c r="AA31" s="98"/>
     </row>
     <row r="32" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="52"/>
-      <c r="C32" s="52"/>
-      <c r="D32" s="52"/>
-      <c r="E32" s="52"/>
-      <c r="F32" s="52"/>
-      <c r="G32" s="52"/>
-      <c r="H32" s="52"/>
-      <c r="I32" s="52"/>
-      <c r="J32" s="52"/>
-      <c r="K32" s="52"/>
-      <c r="L32" s="52"/>
-      <c r="M32" s="52"/>
-      <c r="N32" s="52"/>
-      <c r="O32" s="52"/>
-      <c r="P32" s="52"/>
-      <c r="Q32" s="52"/>
-      <c r="R32" s="34"/>
-      <c r="S32" s="34"/>
-      <c r="T32" s="34"/>
-      <c r="U32" s="34"/>
-      <c r="V32" s="34"/>
-      <c r="W32" s="34"/>
-      <c r="X32" s="34"/>
-      <c r="Y32" s="34"/>
-      <c r="Z32" s="34"/>
-      <c r="AA32" s="34"/>
+      <c r="B32" s="87"/>
+      <c r="C32" s="87"/>
+      <c r="D32" s="87"/>
+      <c r="E32" s="87"/>
+      <c r="F32" s="87"/>
+      <c r="G32" s="87"/>
+      <c r="H32" s="87"/>
+      <c r="I32" s="87"/>
+      <c r="J32" s="87"/>
+      <c r="K32" s="87"/>
+      <c r="L32" s="87"/>
+      <c r="M32" s="87"/>
+      <c r="N32" s="87"/>
+      <c r="O32" s="87"/>
+      <c r="P32" s="87"/>
+      <c r="Q32" s="87"/>
+      <c r="R32" s="98"/>
+      <c r="S32" s="98"/>
+      <c r="T32" s="98"/>
+      <c r="U32" s="98"/>
+      <c r="V32" s="98"/>
+      <c r="W32" s="98"/>
+      <c r="X32" s="98"/>
+      <c r="Y32" s="98"/>
+      <c r="Z32" s="98"/>
+      <c r="AA32" s="98"/>
     </row>
     <row r="33" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="52"/>
-      <c r="C33" s="52"/>
-      <c r="D33" s="52"/>
-      <c r="E33" s="52"/>
-      <c r="F33" s="52"/>
-      <c r="G33" s="52"/>
-      <c r="H33" s="52"/>
-      <c r="I33" s="52"/>
-      <c r="J33" s="52"/>
-      <c r="K33" s="52"/>
-      <c r="L33" s="52"/>
-      <c r="M33" s="52"/>
-      <c r="N33" s="52"/>
-      <c r="O33" s="52"/>
-      <c r="P33" s="52"/>
-      <c r="Q33" s="52"/>
-      <c r="R33" s="34"/>
-      <c r="S33" s="34"/>
-      <c r="T33" s="34"/>
-      <c r="U33" s="34"/>
-      <c r="V33" s="34"/>
-      <c r="W33" s="34"/>
-      <c r="X33" s="34"/>
-      <c r="Y33" s="34"/>
-      <c r="Z33" s="34"/>
-      <c r="AA33" s="34"/>
+      <c r="B33" s="87"/>
+      <c r="C33" s="87"/>
+      <c r="D33" s="87"/>
+      <c r="E33" s="87"/>
+      <c r="F33" s="87"/>
+      <c r="G33" s="87"/>
+      <c r="H33" s="87"/>
+      <c r="I33" s="87"/>
+      <c r="J33" s="87"/>
+      <c r="K33" s="87"/>
+      <c r="L33" s="87"/>
+      <c r="M33" s="87"/>
+      <c r="N33" s="87"/>
+      <c r="O33" s="87"/>
+      <c r="P33" s="87"/>
+      <c r="Q33" s="87"/>
+      <c r="R33" s="98"/>
+      <c r="S33" s="98"/>
+      <c r="T33" s="98"/>
+      <c r="U33" s="98"/>
+      <c r="V33" s="98"/>
+      <c r="W33" s="98"/>
+      <c r="X33" s="98"/>
+      <c r="Y33" s="98"/>
+      <c r="Z33" s="98"/>
+      <c r="AA33" s="98"/>
     </row>
     <row r="34" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="52"/>
-      <c r="C34" s="52"/>
-      <c r="D34" s="52"/>
-      <c r="E34" s="52"/>
-      <c r="F34" s="52"/>
-      <c r="G34" s="52"/>
-      <c r="H34" s="52"/>
-      <c r="I34" s="52"/>
-      <c r="J34" s="52"/>
-      <c r="K34" s="52"/>
-      <c r="L34" s="52"/>
-      <c r="M34" s="52"/>
-      <c r="N34" s="52"/>
-      <c r="O34" s="52"/>
-      <c r="P34" s="52"/>
-      <c r="Q34" s="52"/>
-      <c r="R34" s="34"/>
-      <c r="S34" s="34"/>
-      <c r="T34" s="34"/>
-      <c r="U34" s="34"/>
-      <c r="V34" s="34"/>
-      <c r="W34" s="34"/>
-      <c r="X34" s="34"/>
-      <c r="Y34" s="34"/>
-      <c r="Z34" s="34"/>
-      <c r="AA34" s="34"/>
+      <c r="B34" s="87"/>
+      <c r="C34" s="87"/>
+      <c r="D34" s="87"/>
+      <c r="E34" s="87"/>
+      <c r="F34" s="87"/>
+      <c r="G34" s="87"/>
+      <c r="H34" s="87"/>
+      <c r="I34" s="87"/>
+      <c r="J34" s="87"/>
+      <c r="K34" s="87"/>
+      <c r="L34" s="87"/>
+      <c r="M34" s="87"/>
+      <c r="N34" s="87"/>
+      <c r="O34" s="87"/>
+      <c r="P34" s="87"/>
+      <c r="Q34" s="87"/>
+      <c r="R34" s="98"/>
+      <c r="S34" s="98"/>
+      <c r="T34" s="98"/>
+      <c r="U34" s="98"/>
+      <c r="V34" s="98"/>
+      <c r="W34" s="98"/>
+      <c r="X34" s="98"/>
+      <c r="Y34" s="98"/>
+      <c r="Z34" s="98"/>
+      <c r="AA34" s="98"/>
     </row>
     <row r="35" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="52"/>
-      <c r="C35" s="52"/>
-      <c r="D35" s="52"/>
-      <c r="E35" s="52"/>
-      <c r="F35" s="52"/>
-      <c r="G35" s="52"/>
-      <c r="H35" s="52"/>
-      <c r="I35" s="52"/>
-      <c r="J35" s="52"/>
-      <c r="K35" s="52"/>
-      <c r="L35" s="52"/>
-      <c r="M35" s="52"/>
-      <c r="N35" s="52"/>
-      <c r="O35" s="52"/>
-      <c r="P35" s="52"/>
-      <c r="Q35" s="52"/>
-      <c r="R35" s="34"/>
-      <c r="S35" s="34"/>
-      <c r="T35" s="34"/>
-      <c r="U35" s="34"/>
-      <c r="V35" s="34"/>
-      <c r="W35" s="34"/>
-      <c r="X35" s="34"/>
-      <c r="Y35" s="34"/>
-      <c r="Z35" s="34"/>
-      <c r="AA35" s="34"/>
+      <c r="B35" s="87"/>
+      <c r="C35" s="87"/>
+      <c r="D35" s="87"/>
+      <c r="E35" s="87"/>
+      <c r="F35" s="87"/>
+      <c r="G35" s="87"/>
+      <c r="H35" s="87"/>
+      <c r="I35" s="87"/>
+      <c r="J35" s="87"/>
+      <c r="K35" s="87"/>
+      <c r="L35" s="87"/>
+      <c r="M35" s="87"/>
+      <c r="N35" s="87"/>
+      <c r="O35" s="87"/>
+      <c r="P35" s="87"/>
+      <c r="Q35" s="87"/>
+      <c r="R35" s="98"/>
+      <c r="S35" s="98"/>
+      <c r="T35" s="98"/>
+      <c r="U35" s="98"/>
+      <c r="V35" s="98"/>
+      <c r="W35" s="98"/>
+      <c r="X35" s="98"/>
+      <c r="Y35" s="98"/>
+      <c r="Z35" s="98"/>
+      <c r="AA35" s="98"/>
     </row>
     <row r="36" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="52"/>
-      <c r="C36" s="52"/>
-      <c r="D36" s="52"/>
-      <c r="E36" s="52"/>
-      <c r="F36" s="52"/>
-      <c r="G36" s="52"/>
-      <c r="H36" s="52"/>
-      <c r="I36" s="52"/>
-      <c r="J36" s="52"/>
-      <c r="K36" s="52"/>
-      <c r="L36" s="52"/>
-      <c r="M36" s="52"/>
-      <c r="N36" s="52"/>
-      <c r="O36" s="52"/>
-      <c r="P36" s="52"/>
-      <c r="Q36" s="52"/>
-      <c r="R36" s="34"/>
-      <c r="S36" s="34"/>
-      <c r="T36" s="34"/>
-      <c r="U36" s="34"/>
-      <c r="V36" s="34"/>
-      <c r="W36" s="34"/>
-      <c r="X36" s="34"/>
-      <c r="Y36" s="34"/>
-      <c r="Z36" s="34"/>
-      <c r="AA36" s="34"/>
+      <c r="B36" s="87"/>
+      <c r="C36" s="87"/>
+      <c r="D36" s="87"/>
+      <c r="E36" s="87"/>
+      <c r="F36" s="87"/>
+      <c r="G36" s="87"/>
+      <c r="H36" s="87"/>
+      <c r="I36" s="87"/>
+      <c r="J36" s="87"/>
+      <c r="K36" s="87"/>
+      <c r="L36" s="87"/>
+      <c r="M36" s="87"/>
+      <c r="N36" s="87"/>
+      <c r="O36" s="87"/>
+      <c r="P36" s="87"/>
+      <c r="Q36" s="87"/>
+      <c r="R36" s="98"/>
+      <c r="S36" s="98"/>
+      <c r="T36" s="98"/>
+      <c r="U36" s="98"/>
+      <c r="V36" s="98"/>
+      <c r="W36" s="98"/>
+      <c r="X36" s="98"/>
+      <c r="Y36" s="98"/>
+      <c r="Z36" s="98"/>
+      <c r="AA36" s="98"/>
     </row>
     <row r="37" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="52"/>
-      <c r="C37" s="52"/>
-      <c r="D37" s="52"/>
-      <c r="E37" s="52"/>
-      <c r="F37" s="52"/>
-      <c r="G37" s="52"/>
-      <c r="H37" s="52"/>
-      <c r="I37" s="52"/>
-      <c r="J37" s="52"/>
-      <c r="K37" s="52"/>
-      <c r="L37" s="52"/>
-      <c r="M37" s="52"/>
-      <c r="N37" s="52"/>
-      <c r="O37" s="52"/>
-      <c r="P37" s="52"/>
-      <c r="Q37" s="52"/>
-      <c r="R37" s="34"/>
-      <c r="S37" s="34"/>
-      <c r="T37" s="34"/>
-      <c r="U37" s="34"/>
-      <c r="V37" s="34"/>
-      <c r="W37" s="34"/>
-      <c r="X37" s="34"/>
-      <c r="Y37" s="34"/>
-      <c r="Z37" s="34"/>
-      <c r="AA37" s="34"/>
+      <c r="B37" s="87"/>
+      <c r="C37" s="87"/>
+      <c r="D37" s="87"/>
+      <c r="E37" s="87"/>
+      <c r="F37" s="87"/>
+      <c r="G37" s="87"/>
+      <c r="H37" s="87"/>
+      <c r="I37" s="87"/>
+      <c r="J37" s="87"/>
+      <c r="K37" s="87"/>
+      <c r="L37" s="87"/>
+      <c r="M37" s="87"/>
+      <c r="N37" s="87"/>
+      <c r="O37" s="87"/>
+      <c r="P37" s="87"/>
+      <c r="Q37" s="87"/>
+      <c r="R37" s="98"/>
+      <c r="S37" s="98"/>
+      <c r="T37" s="98"/>
+      <c r="U37" s="98"/>
+      <c r="V37" s="98"/>
+      <c r="W37" s="98"/>
+      <c r="X37" s="98"/>
+      <c r="Y37" s="98"/>
+      <c r="Z37" s="98"/>
+      <c r="AA37" s="98"/>
     </row>
     <row r="38" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="52"/>
-      <c r="C38" s="52"/>
-      <c r="D38" s="52"/>
-      <c r="E38" s="52"/>
-      <c r="F38" s="52"/>
-      <c r="G38" s="52"/>
-      <c r="H38" s="52"/>
-      <c r="I38" s="52"/>
-      <c r="J38" s="52"/>
-      <c r="K38" s="52"/>
-      <c r="L38" s="52"/>
-      <c r="M38" s="52"/>
-      <c r="N38" s="52"/>
-      <c r="O38" s="52"/>
-      <c r="P38" s="52"/>
-      <c r="Q38" s="52"/>
-      <c r="R38" s="34"/>
-      <c r="S38" s="34"/>
-      <c r="T38" s="34"/>
-      <c r="U38" s="34"/>
-      <c r="V38" s="34"/>
-      <c r="W38" s="34"/>
-      <c r="X38" s="34"/>
-      <c r="Y38" s="34"/>
-      <c r="Z38" s="34"/>
-      <c r="AA38" s="34"/>
+      <c r="B38" s="87"/>
+      <c r="C38" s="87"/>
+      <c r="D38" s="87"/>
+      <c r="E38" s="87"/>
+      <c r="F38" s="87"/>
+      <c r="G38" s="87"/>
+      <c r="H38" s="87"/>
+      <c r="I38" s="87"/>
+      <c r="J38" s="87"/>
+      <c r="K38" s="87"/>
+      <c r="L38" s="87"/>
+      <c r="M38" s="87"/>
+      <c r="N38" s="87"/>
+      <c r="O38" s="87"/>
+      <c r="P38" s="87"/>
+      <c r="Q38" s="87"/>
+      <c r="R38" s="98"/>
+      <c r="S38" s="98"/>
+      <c r="T38" s="98"/>
+      <c r="U38" s="98"/>
+      <c r="V38" s="98"/>
+      <c r="W38" s="98"/>
+      <c r="X38" s="98"/>
+      <c r="Y38" s="98"/>
+      <c r="Z38" s="98"/>
+      <c r="AA38" s="98"/>
     </row>
     <row r="39" spans="2:27" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="52"/>
-      <c r="C39" s="52"/>
-      <c r="D39" s="52"/>
-      <c r="E39" s="52"/>
-      <c r="F39" s="52"/>
-      <c r="G39" s="52"/>
-      <c r="H39" s="52"/>
-      <c r="I39" s="52"/>
-      <c r="J39" s="52"/>
-      <c r="K39" s="52"/>
-      <c r="L39" s="52"/>
-      <c r="M39" s="52"/>
-      <c r="N39" s="52"/>
-      <c r="O39" s="52"/>
-      <c r="P39" s="52"/>
-      <c r="Q39" s="52"/>
-      <c r="R39" s="34"/>
-      <c r="S39" s="34"/>
-      <c r="T39" s="34"/>
-      <c r="U39" s="34"/>
-      <c r="V39" s="34"/>
-      <c r="W39" s="34"/>
-      <c r="X39" s="34"/>
-      <c r="Y39" s="34"/>
-      <c r="Z39" s="34"/>
-      <c r="AA39" s="34"/>
+      <c r="B39" s="87"/>
+      <c r="C39" s="87"/>
+      <c r="D39" s="87"/>
+      <c r="E39" s="87"/>
+      <c r="F39" s="87"/>
+      <c r="G39" s="87"/>
+      <c r="H39" s="87"/>
+      <c r="I39" s="87"/>
+      <c r="J39" s="87"/>
+      <c r="K39" s="87"/>
+      <c r="L39" s="87"/>
+      <c r="M39" s="87"/>
+      <c r="N39" s="87"/>
+      <c r="O39" s="87"/>
+      <c r="P39" s="87"/>
+      <c r="Q39" s="87"/>
+      <c r="R39" s="98"/>
+      <c r="S39" s="98"/>
+      <c r="T39" s="98"/>
+      <c r="U39" s="98"/>
+      <c r="V39" s="98"/>
+      <c r="W39" s="98"/>
+      <c r="X39" s="98"/>
+      <c r="Y39" s="98"/>
+      <c r="Z39" s="98"/>
+      <c r="AA39" s="98"/>
     </row>
     <row r="40" spans="2:27" ht="6.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="35" t="s">
+      <c r="B40" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="C40" s="35"/>
-      <c r="D40" s="35"/>
-      <c r="E40" s="35"/>
-      <c r="F40" s="35"/>
-      <c r="G40" s="35"/>
-      <c r="H40" s="35"/>
-      <c r="I40" s="35"/>
-      <c r="J40" s="35"/>
-      <c r="K40" s="35"/>
-      <c r="L40" s="35"/>
-      <c r="M40" s="35"/>
-      <c r="N40" s="35"/>
-      <c r="O40" s="35"/>
-      <c r="P40" s="35"/>
-      <c r="Q40" s="35"/>
-      <c r="R40" s="35"/>
-      <c r="S40" s="35"/>
-      <c r="T40" s="35"/>
-      <c r="U40" s="35"/>
-      <c r="V40" s="35"/>
-      <c r="W40" s="35"/>
-      <c r="X40" s="35"/>
-      <c r="Y40" s="35"/>
-      <c r="Z40" s="35"/>
-      <c r="AA40" s="35"/>
+      <c r="C40" s="31"/>
+      <c r="D40" s="31"/>
+      <c r="E40" s="31"/>
+      <c r="F40" s="31"/>
+      <c r="G40" s="31"/>
+      <c r="H40" s="31"/>
+      <c r="I40" s="31"/>
+      <c r="J40" s="31"/>
+      <c r="K40" s="31"/>
+      <c r="L40" s="31"/>
+      <c r="M40" s="31"/>
+      <c r="N40" s="31"/>
+      <c r="O40" s="31"/>
+      <c r="P40" s="31"/>
+      <c r="Q40" s="31"/>
+      <c r="R40" s="31"/>
+      <c r="S40" s="31"/>
+      <c r="T40" s="31"/>
+      <c r="U40" s="31"/>
+      <c r="V40" s="31"/>
+      <c r="W40" s="31"/>
+      <c r="X40" s="31"/>
+      <c r="Y40" s="31"/>
+      <c r="Z40" s="31"/>
+      <c r="AA40" s="31"/>
     </row>
     <row r="41" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="25" t="s">
+      <c r="B41" s="109" t="s">
         <v>19</v>
       </c>
-      <c r="C41" s="26"/>
-      <c r="D41" s="26"/>
-      <c r="E41" s="26"/>
-      <c r="F41" s="26"/>
-      <c r="G41" s="26"/>
-      <c r="H41" s="26"/>
-      <c r="I41" s="26"/>
-      <c r="J41" s="26"/>
-      <c r="K41" s="26"/>
-      <c r="L41" s="26"/>
-      <c r="M41" s="26"/>
-      <c r="N41" s="26"/>
-      <c r="O41" s="26"/>
-      <c r="P41" s="26"/>
-      <c r="Q41" s="26"/>
-      <c r="R41" s="26"/>
-      <c r="S41" s="26"/>
-      <c r="T41" s="26"/>
-      <c r="U41" s="26"/>
-      <c r="V41" s="26"/>
-      <c r="W41" s="26"/>
-      <c r="X41" s="26"/>
-      <c r="Y41" s="26"/>
-      <c r="Z41" s="26"/>
-      <c r="AA41" s="27"/>
+      <c r="C41" s="110"/>
+      <c r="D41" s="110"/>
+      <c r="E41" s="110"/>
+      <c r="F41" s="110"/>
+      <c r="G41" s="110"/>
+      <c r="H41" s="110"/>
+      <c r="I41" s="110"/>
+      <c r="J41" s="110"/>
+      <c r="K41" s="110"/>
+      <c r="L41" s="110"/>
+      <c r="M41" s="110"/>
+      <c r="N41" s="110"/>
+      <c r="O41" s="110"/>
+      <c r="P41" s="110"/>
+      <c r="Q41" s="110"/>
+      <c r="R41" s="110"/>
+      <c r="S41" s="110"/>
+      <c r="T41" s="110"/>
+      <c r="U41" s="110"/>
+      <c r="V41" s="110"/>
+      <c r="W41" s="110"/>
+      <c r="X41" s="110"/>
+      <c r="Y41" s="110"/>
+      <c r="Z41" s="110"/>
+      <c r="AA41" s="111"/>
     </row>
     <row r="42" spans="2:27" ht="36.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="108" t="s">
+      <c r="B42" s="50" t="s">
         <v>10</v>
       </c>
-      <c r="C42" s="103"/>
-      <c r="D42" s="28" t="s">
+      <c r="C42" s="43"/>
+      <c r="D42" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="E42" s="29"/>
-      <c r="F42" s="28" t="s">
+      <c r="E42" s="52"/>
+      <c r="F42" s="36" t="s">
         <v>54</v>
       </c>
-      <c r="G42" s="29"/>
-      <c r="H42" s="28" t="s">
+      <c r="G42" s="52"/>
+      <c r="H42" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="I42" s="29"/>
-      <c r="J42" s="28" t="s">
+      <c r="I42" s="52"/>
+      <c r="J42" s="36" t="s">
         <v>56</v>
       </c>
-      <c r="K42" s="29"/>
-      <c r="L42" s="28" t="s">
+      <c r="K42" s="52"/>
+      <c r="L42" s="36" t="s">
         <v>57</v>
       </c>
-      <c r="M42" s="29"/>
-      <c r="N42" s="28" t="s">
+      <c r="M42" s="52"/>
+      <c r="N42" s="36" t="s">
         <v>58</v>
       </c>
-      <c r="O42" s="32"/>
-      <c r="P42" s="28" t="s">
+      <c r="O42" s="37"/>
+      <c r="P42" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="Q42" s="32"/>
-      <c r="R42" s="28" t="s">
+      <c r="Q42" s="37"/>
+      <c r="R42" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="S42" s="32"/>
-      <c r="T42" s="28" t="s">
+      <c r="S42" s="37"/>
+      <c r="T42" s="36" t="s">
         <v>61</v>
       </c>
-      <c r="U42" s="32"/>
-      <c r="V42" s="28" t="s">
+      <c r="U42" s="37"/>
+      <c r="V42" s="36" t="s">
         <v>62</v>
       </c>
-      <c r="W42" s="32"/>
-      <c r="X42" s="28" t="s">
+      <c r="W42" s="37"/>
+      <c r="X42" s="36" t="s">
         <v>63</v>
       </c>
-      <c r="Y42" s="32"/>
-      <c r="Z42" s="28" t="s">
+      <c r="Y42" s="37"/>
+      <c r="Z42" s="36" t="s">
         <v>64</v>
       </c>
-      <c r="AA42" s="32"/>
+      <c r="AA42" s="37"/>
     </row>
     <row r="43" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="109"/>
-      <c r="C43" s="105"/>
+      <c r="B43" s="51"/>
+      <c r="C43" s="45"/>
       <c r="D43" s="11" t="s">
         <v>11</v>
       </c>
@@ -9850,8 +9846,8 @@
       </c>
     </row>
     <row r="44" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="106"/>
-      <c r="C44" s="107"/>
+      <c r="B44" s="46"/>
+      <c r="C44" s="47"/>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
@@ -9878,60 +9874,60 @@
       <c r="AA44" s="3"/>
     </row>
     <row r="45" spans="2:27" ht="36.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="102" t="s">
+      <c r="B45" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="C45" s="103"/>
-      <c r="D45" s="28" t="s">
+      <c r="C45" s="43"/>
+      <c r="D45" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="E45" s="29"/>
-      <c r="F45" s="28" t="s">
+      <c r="E45" s="52"/>
+      <c r="F45" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="G45" s="29"/>
-      <c r="H45" s="28" t="s">
+      <c r="G45" s="52"/>
+      <c r="H45" s="36" t="s">
         <v>26</v>
       </c>
-      <c r="I45" s="29"/>
-      <c r="J45" s="28" t="s">
+      <c r="I45" s="52"/>
+      <c r="J45" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="K45" s="29"/>
-      <c r="L45" s="28" t="s">
+      <c r="K45" s="52"/>
+      <c r="L45" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="M45" s="32"/>
-      <c r="N45" s="28" t="s">
+      <c r="M45" s="37"/>
+      <c r="N45" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="O45" s="32"/>
-      <c r="P45" s="28" t="s">
+      <c r="O45" s="37"/>
+      <c r="P45" s="36" t="s">
         <v>33</v>
       </c>
-      <c r="Q45" s="32"/>
-      <c r="R45" s="28" t="s">
+      <c r="Q45" s="37"/>
+      <c r="R45" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="S45" s="32"/>
-      <c r="T45" s="28" t="s">
+      <c r="S45" s="37"/>
+      <c r="T45" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="U45" s="32"/>
-      <c r="V45" s="28" t="s">
+      <c r="U45" s="37"/>
+      <c r="V45" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="W45" s="32"/>
-      <c r="X45" s="30" t="s">
+      <c r="W45" s="37"/>
+      <c r="X45" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="Y45" s="31"/>
-      <c r="Z45" s="31"/>
-      <c r="AA45" s="31"/>
+      <c r="Y45" s="39"/>
+      <c r="Z45" s="39"/>
+      <c r="AA45" s="39"/>
     </row>
     <row r="46" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="104"/>
-      <c r="C46" s="105"/>
+      <c r="B46" s="44"/>
+      <c r="C46" s="45"/>
       <c r="D46" s="11" t="s">
         <v>11</v>
       </c>
@@ -10006,8 +10002,8 @@
       </c>
     </row>
     <row r="47" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="106"/>
-      <c r="C47" s="107"/>
+      <c r="B47" s="46"/>
+      <c r="C47" s="47"/>
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
@@ -10036,62 +10032,62 @@
       <c r="AA47" s="3"/>
     </row>
     <row r="48" spans="2:27" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="102" t="s">
+      <c r="B48" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="C48" s="103"/>
-      <c r="D48" s="30" t="s">
+      <c r="C48" s="43"/>
+      <c r="D48" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="E48" s="31"/>
-      <c r="F48" s="30" t="s">
+      <c r="E48" s="39"/>
+      <c r="F48" s="38" t="s">
         <v>66</v>
       </c>
-      <c r="G48" s="31"/>
-      <c r="H48" s="30" t="s">
+      <c r="G48" s="39"/>
+      <c r="H48" s="38" t="s">
         <v>67</v>
       </c>
-      <c r="I48" s="31"/>
-      <c r="J48" s="30" t="s">
+      <c r="I48" s="39"/>
+      <c r="J48" s="38" t="s">
         <v>68</v>
       </c>
-      <c r="K48" s="31"/>
-      <c r="L48" s="30" t="s">
+      <c r="K48" s="39"/>
+      <c r="L48" s="38" t="s">
         <v>68</v>
       </c>
-      <c r="M48" s="31"/>
-      <c r="N48" s="30" t="s">
+      <c r="M48" s="39"/>
+      <c r="N48" s="38" t="s">
         <v>69</v>
       </c>
-      <c r="O48" s="31"/>
-      <c r="P48" s="28" t="s">
+      <c r="O48" s="39"/>
+      <c r="P48" s="36" t="s">
         <v>70</v>
       </c>
-      <c r="Q48" s="29"/>
-      <c r="R48" s="89" t="s">
+      <c r="Q48" s="52"/>
+      <c r="R48" s="48" t="s">
         <v>71</v>
       </c>
-      <c r="S48" s="90"/>
-      <c r="T48" s="100" t="s">
+      <c r="S48" s="49"/>
+      <c r="T48" s="40" t="s">
         <v>72</v>
       </c>
-      <c r="U48" s="101"/>
-      <c r="V48" s="100" t="s">
+      <c r="U48" s="41"/>
+      <c r="V48" s="40" t="s">
         <v>73</v>
       </c>
-      <c r="W48" s="101"/>
-      <c r="X48" s="100" t="s">
+      <c r="W48" s="41"/>
+      <c r="X48" s="40" t="s">
         <v>74</v>
       </c>
-      <c r="Y48" s="101"/>
-      <c r="Z48" s="28" t="s">
+      <c r="Y48" s="41"/>
+      <c r="Z48" s="36" t="s">
         <v>75</v>
       </c>
-      <c r="AA48" s="29"/>
+      <c r="AA48" s="52"/>
     </row>
     <row r="49" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="104"/>
-      <c r="C49" s="105"/>
+      <c r="B49" s="44"/>
+      <c r="C49" s="45"/>
       <c r="D49" s="11" t="s">
         <v>11</v>
       </c>
@@ -10166,8 +10162,8 @@
       </c>
     </row>
     <row r="50" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="104"/>
-      <c r="C50" s="105"/>
+      <c r="B50" s="44"/>
+      <c r="C50" s="45"/>
       <c r="D50" s="3"/>
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
@@ -10194,58 +10190,58 @@
       <c r="AA50" s="3"/>
     </row>
     <row r="51" spans="2:27" ht="36.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B51" s="104"/>
-      <c r="C51" s="105"/>
-      <c r="D51" s="30" t="s">
+      <c r="B51" s="44"/>
+      <c r="C51" s="45"/>
+      <c r="D51" s="38" t="s">
         <v>76</v>
       </c>
-      <c r="E51" s="31"/>
-      <c r="F51" s="30" t="s">
+      <c r="E51" s="39"/>
+      <c r="F51" s="38" t="s">
         <v>77</v>
       </c>
-      <c r="G51" s="31"/>
-      <c r="H51" s="30" t="s">
+      <c r="G51" s="39"/>
+      <c r="H51" s="38" t="s">
         <v>78</v>
       </c>
-      <c r="I51" s="31"/>
-      <c r="J51" s="30" t="s">
+      <c r="I51" s="39"/>
+      <c r="J51" s="38" t="s">
         <v>79</v>
       </c>
-      <c r="K51" s="31"/>
-      <c r="L51" s="89" t="s">
+      <c r="K51" s="39"/>
+      <c r="L51" s="48" t="s">
         <v>80</v>
       </c>
-      <c r="M51" s="90"/>
-      <c r="N51" s="30" t="s">
+      <c r="M51" s="49"/>
+      <c r="N51" s="38" t="s">
         <v>81</v>
       </c>
-      <c r="O51" s="31"/>
-      <c r="P51" s="89" t="s">
+      <c r="O51" s="39"/>
+      <c r="P51" s="48" t="s">
         <v>82</v>
       </c>
-      <c r="Q51" s="90"/>
-      <c r="R51" s="30" t="s">
+      <c r="Q51" s="49"/>
+      <c r="R51" s="38" t="s">
         <v>83</v>
       </c>
-      <c r="S51" s="31"/>
-      <c r="T51" s="98" t="s">
+      <c r="S51" s="39"/>
+      <c r="T51" s="63" t="s">
         <v>84</v>
       </c>
-      <c r="U51" s="99"/>
-      <c r="V51" s="28" t="s">
+      <c r="U51" s="64"/>
+      <c r="V51" s="36" t="s">
         <v>85</v>
       </c>
-      <c r="W51" s="32"/>
-      <c r="X51" s="28" t="s">
+      <c r="W51" s="37"/>
+      <c r="X51" s="36" t="s">
         <v>86</v>
       </c>
-      <c r="Y51" s="32"/>
-      <c r="Z51" s="97"/>
-      <c r="AA51" s="65"/>
+      <c r="Y51" s="37"/>
+      <c r="Z51" s="61"/>
+      <c r="AA51" s="62"/>
     </row>
     <row r="52" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="104"/>
-      <c r="C52" s="105"/>
+      <c r="B52" s="44"/>
+      <c r="C52" s="45"/>
       <c r="D52" s="11" t="s">
         <v>11</v>
       </c>
@@ -10316,8 +10312,8 @@
       <c r="AA52" s="11"/>
     </row>
     <row r="53" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B53" s="106"/>
-      <c r="C53" s="107"/>
+      <c r="B53" s="46"/>
+      <c r="C53" s="47"/>
       <c r="D53" s="3"/>
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
@@ -10344,84 +10340,84 @@
       <c r="AA53" s="3"/>
     </row>
     <row r="54" spans="2:27" ht="6.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B54" s="35"/>
-      <c r="C54" s="35"/>
-      <c r="D54" s="35"/>
-      <c r="E54" s="35"/>
-      <c r="F54" s="35"/>
-      <c r="G54" s="35"/>
-      <c r="H54" s="35"/>
-      <c r="I54" s="35"/>
-      <c r="J54" s="35"/>
-      <c r="K54" s="35"/>
-      <c r="L54" s="35"/>
-      <c r="M54" s="35"/>
-      <c r="N54" s="35"/>
-      <c r="O54" s="35"/>
-      <c r="P54" s="35"/>
-      <c r="Q54" s="35"/>
-      <c r="R54" s="35"/>
-      <c r="S54" s="35"/>
-      <c r="T54" s="35"/>
-      <c r="U54" s="35"/>
-      <c r="V54" s="35"/>
-      <c r="W54" s="35"/>
-      <c r="X54" s="35"/>
-      <c r="Y54" s="35"/>
-      <c r="Z54" s="35"/>
-      <c r="AA54" s="35"/>
+      <c r="B54" s="31"/>
+      <c r="C54" s="31"/>
+      <c r="D54" s="31"/>
+      <c r="E54" s="31"/>
+      <c r="F54" s="31"/>
+      <c r="G54" s="31"/>
+      <c r="H54" s="31"/>
+      <c r="I54" s="31"/>
+      <c r="J54" s="31"/>
+      <c r="K54" s="31"/>
+      <c r="L54" s="31"/>
+      <c r="M54" s="31"/>
+      <c r="N54" s="31"/>
+      <c r="O54" s="31"/>
+      <c r="P54" s="31"/>
+      <c r="Q54" s="31"/>
+      <c r="R54" s="31"/>
+      <c r="S54" s="31"/>
+      <c r="T54" s="31"/>
+      <c r="U54" s="31"/>
+      <c r="V54" s="31"/>
+      <c r="W54" s="31"/>
+      <c r="X54" s="31"/>
+      <c r="Y54" s="31"/>
+      <c r="Z54" s="31"/>
+      <c r="AA54" s="31"/>
     </row>
     <row r="55" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="88" t="s">
+      <c r="B55" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="C55" s="88"/>
-      <c r="D55" s="88"/>
-      <c r="E55" s="88"/>
-      <c r="F55" s="88"/>
-      <c r="G55" s="88"/>
-      <c r="H55" s="88"/>
-      <c r="I55" s="88"/>
-      <c r="J55" s="88"/>
-      <c r="K55" s="88"/>
-      <c r="L55" s="88"/>
-      <c r="M55" s="88"/>
-      <c r="N55" s="88"/>
-      <c r="O55" s="88"/>
-      <c r="P55" s="88"/>
-      <c r="Q55" s="88"/>
-      <c r="R55" s="88"/>
-      <c r="S55" s="88"/>
-      <c r="T55" s="88"/>
-      <c r="U55" s="88"/>
-      <c r="V55" s="88"/>
-      <c r="W55" s="88"/>
-      <c r="X55" s="88"/>
-      <c r="Y55" s="88"/>
-      <c r="Z55" s="88"/>
-      <c r="AA55" s="88"/>
+      <c r="C55" s="54"/>
+      <c r="D55" s="54"/>
+      <c r="E55" s="54"/>
+      <c r="F55" s="54"/>
+      <c r="G55" s="54"/>
+      <c r="H55" s="54"/>
+      <c r="I55" s="54"/>
+      <c r="J55" s="54"/>
+      <c r="K55" s="54"/>
+      <c r="L55" s="54"/>
+      <c r="M55" s="54"/>
+      <c r="N55" s="54"/>
+      <c r="O55" s="54"/>
+      <c r="P55" s="54"/>
+      <c r="Q55" s="54"/>
+      <c r="R55" s="54"/>
+      <c r="S55" s="54"/>
+      <c r="T55" s="54"/>
+      <c r="U55" s="54"/>
+      <c r="V55" s="54"/>
+      <c r="W55" s="54"/>
+      <c r="X55" s="54"/>
+      <c r="Y55" s="54"/>
+      <c r="Z55" s="54"/>
+      <c r="AA55" s="54"/>
     </row>
     <row r="56" spans="2:27" ht="36.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="86" t="s">
+      <c r="B56" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="C56" s="86"/>
-      <c r="D56" s="86"/>
-      <c r="E56" s="86"/>
-      <c r="F56" s="86" t="s">
+      <c r="C56" s="32"/>
+      <c r="D56" s="32"/>
+      <c r="E56" s="32"/>
+      <c r="F56" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="G56" s="86"/>
-      <c r="H56" s="86"/>
-      <c r="I56" s="110" t="s">
+      <c r="G56" s="32"/>
+      <c r="H56" s="32"/>
+      <c r="I56" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="J56" s="114"/>
+      <c r="J56" s="35"/>
       <c r="K56" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="L56" s="16" t="s">
         <v>89</v>
-      </c>
-      <c r="L56" s="16" t="s">
-        <v>90</v>
       </c>
       <c r="M56" s="17" t="s">
         <v>3</v>
@@ -10429,26 +10425,26 @@
       <c r="N56" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="O56" s="86" t="s">
+      <c r="O56" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="P56" s="86"/>
-      <c r="Q56" s="86"/>
-      <c r="R56" s="86"/>
-      <c r="S56" s="86" t="s">
+      <c r="P56" s="32"/>
+      <c r="Q56" s="32"/>
+      <c r="R56" s="32"/>
+      <c r="S56" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="T56" s="86"/>
-      <c r="U56" s="86"/>
-      <c r="V56" s="110" t="s">
+      <c r="T56" s="32"/>
+      <c r="U56" s="32"/>
+      <c r="V56" s="33" t="s">
         <v>49</v>
       </c>
-      <c r="W56" s="111"/>
+      <c r="W56" s="34"/>
       <c r="X56" s="16" t="s">
         <v>43</v>
       </c>
       <c r="Y56" s="16" t="s">
-        <v>88</v>
+        <v>3</v>
       </c>
       <c r="Z56" s="16" t="s">
         <v>3</v>
@@ -10458,206 +10454,206 @@
       </c>
     </row>
     <row r="57" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B57" s="83"/>
-      <c r="C57" s="84"/>
-      <c r="D57" s="84"/>
-      <c r="E57" s="85"/>
-      <c r="F57" s="83"/>
-      <c r="G57" s="84"/>
-      <c r="H57" s="85"/>
-      <c r="I57" s="112"/>
-      <c r="J57" s="113"/>
+      <c r="B57" s="27"/>
+      <c r="C57" s="28"/>
+      <c r="D57" s="28"/>
+      <c r="E57" s="29"/>
+      <c r="F57" s="27"/>
+      <c r="G57" s="28"/>
+      <c r="H57" s="29"/>
+      <c r="I57" s="25"/>
+      <c r="J57" s="26"/>
       <c r="K57" s="15"/>
       <c r="L57" s="18"/>
       <c r="M57" s="19"/>
       <c r="N57" s="20"/>
-      <c r="O57" s="83"/>
-      <c r="P57" s="84"/>
-      <c r="Q57" s="84"/>
-      <c r="R57" s="85"/>
-      <c r="S57" s="83"/>
-      <c r="T57" s="84"/>
-      <c r="U57" s="85"/>
-      <c r="V57" s="112"/>
-      <c r="W57" s="113"/>
+      <c r="O57" s="27"/>
+      <c r="P57" s="28"/>
+      <c r="Q57" s="28"/>
+      <c r="R57" s="29"/>
+      <c r="S57" s="27"/>
+      <c r="T57" s="28"/>
+      <c r="U57" s="29"/>
+      <c r="V57" s="25"/>
+      <c r="W57" s="26"/>
       <c r="X57" s="15"/>
       <c r="Y57" s="21"/>
       <c r="Z57" s="22"/>
       <c r="AA57" s="22"/>
     </row>
     <row r="58" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B58" s="87"/>
-      <c r="C58" s="87"/>
-      <c r="D58" s="87"/>
-      <c r="E58" s="87"/>
-      <c r="F58" s="87"/>
-      <c r="G58" s="87"/>
-      <c r="H58" s="87"/>
-      <c r="I58" s="112"/>
-      <c r="J58" s="113"/>
+      <c r="B58" s="30"/>
+      <c r="C58" s="30"/>
+      <c r="D58" s="30"/>
+      <c r="E58" s="30"/>
+      <c r="F58" s="30"/>
+      <c r="G58" s="30"/>
+      <c r="H58" s="30"/>
+      <c r="I58" s="25"/>
+      <c r="J58" s="26"/>
       <c r="K58" s="15"/>
       <c r="L58" s="18"/>
       <c r="M58" s="19"/>
       <c r="N58" s="20"/>
-      <c r="O58" s="83"/>
-      <c r="P58" s="84"/>
-      <c r="Q58" s="84"/>
-      <c r="R58" s="85"/>
-      <c r="S58" s="83"/>
-      <c r="T58" s="84"/>
-      <c r="U58" s="85"/>
-      <c r="V58" s="112"/>
-      <c r="W58" s="113"/>
+      <c r="O58" s="27"/>
+      <c r="P58" s="28"/>
+      <c r="Q58" s="28"/>
+      <c r="R58" s="29"/>
+      <c r="S58" s="27"/>
+      <c r="T58" s="28"/>
+      <c r="U58" s="29"/>
+      <c r="V58" s="25"/>
+      <c r="W58" s="26"/>
       <c r="X58" s="15"/>
       <c r="Y58" s="21"/>
       <c r="Z58" s="22"/>
       <c r="AA58" s="22"/>
     </row>
     <row r="59" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="87"/>
-      <c r="C59" s="87"/>
-      <c r="D59" s="87"/>
-      <c r="E59" s="87"/>
-      <c r="F59" s="83"/>
-      <c r="G59" s="84"/>
-      <c r="H59" s="85"/>
-      <c r="I59" s="112"/>
-      <c r="J59" s="113"/>
+      <c r="B59" s="30"/>
+      <c r="C59" s="30"/>
+      <c r="D59" s="30"/>
+      <c r="E59" s="30"/>
+      <c r="F59" s="27"/>
+      <c r="G59" s="28"/>
+      <c r="H59" s="29"/>
+      <c r="I59" s="25"/>
+      <c r="J59" s="26"/>
       <c r="K59" s="15"/>
       <c r="L59" s="22"/>
       <c r="M59" s="19"/>
       <c r="N59" s="20"/>
-      <c r="O59" s="83"/>
-      <c r="P59" s="84"/>
-      <c r="Q59" s="84"/>
-      <c r="R59" s="85"/>
-      <c r="S59" s="83"/>
-      <c r="T59" s="84"/>
-      <c r="U59" s="85"/>
-      <c r="V59" s="112"/>
-      <c r="W59" s="113"/>
+      <c r="O59" s="27"/>
+      <c r="P59" s="28"/>
+      <c r="Q59" s="28"/>
+      <c r="R59" s="29"/>
+      <c r="S59" s="27"/>
+      <c r="T59" s="28"/>
+      <c r="U59" s="29"/>
+      <c r="V59" s="25"/>
+      <c r="W59" s="26"/>
       <c r="X59" s="15"/>
       <c r="Y59" s="21"/>
       <c r="Z59" s="22"/>
       <c r="AA59" s="22"/>
     </row>
     <row r="60" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="87"/>
-      <c r="C60" s="87"/>
-      <c r="D60" s="87"/>
-      <c r="E60" s="87"/>
-      <c r="F60" s="87"/>
-      <c r="G60" s="87"/>
-      <c r="H60" s="87"/>
-      <c r="I60" s="112"/>
-      <c r="J60" s="113"/>
+      <c r="B60" s="30"/>
+      <c r="C60" s="30"/>
+      <c r="D60" s="30"/>
+      <c r="E60" s="30"/>
+      <c r="F60" s="30"/>
+      <c r="G60" s="30"/>
+      <c r="H60" s="30"/>
+      <c r="I60" s="25"/>
+      <c r="J60" s="26"/>
       <c r="K60" s="15"/>
       <c r="L60" s="18"/>
       <c r="M60" s="19"/>
       <c r="N60" s="20"/>
-      <c r="O60" s="83"/>
-      <c r="P60" s="84"/>
-      <c r="Q60" s="84"/>
-      <c r="R60" s="85"/>
-      <c r="S60" s="83"/>
-      <c r="T60" s="84"/>
-      <c r="U60" s="85"/>
-      <c r="V60" s="112"/>
-      <c r="W60" s="113"/>
+      <c r="O60" s="27"/>
+      <c r="P60" s="28"/>
+      <c r="Q60" s="28"/>
+      <c r="R60" s="29"/>
+      <c r="S60" s="27"/>
+      <c r="T60" s="28"/>
+      <c r="U60" s="29"/>
+      <c r="V60" s="25"/>
+      <c r="W60" s="26"/>
       <c r="X60" s="15"/>
       <c r="Y60" s="21"/>
       <c r="Z60" s="22"/>
       <c r="AA60" s="22"/>
     </row>
     <row r="61" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="83"/>
-      <c r="C61" s="84"/>
-      <c r="D61" s="84"/>
-      <c r="E61" s="85"/>
-      <c r="F61" s="83"/>
-      <c r="G61" s="84"/>
-      <c r="H61" s="85"/>
-      <c r="I61" s="112"/>
-      <c r="J61" s="113"/>
+      <c r="B61" s="27"/>
+      <c r="C61" s="28"/>
+      <c r="D61" s="28"/>
+      <c r="E61" s="29"/>
+      <c r="F61" s="27"/>
+      <c r="G61" s="28"/>
+      <c r="H61" s="29"/>
+      <c r="I61" s="25"/>
+      <c r="J61" s="26"/>
       <c r="K61" s="15"/>
       <c r="L61" s="22"/>
       <c r="M61" s="19"/>
       <c r="N61" s="23"/>
-      <c r="O61" s="83"/>
-      <c r="P61" s="84"/>
-      <c r="Q61" s="84"/>
-      <c r="R61" s="85"/>
-      <c r="S61" s="83"/>
-      <c r="T61" s="84"/>
-      <c r="U61" s="85"/>
-      <c r="V61" s="112"/>
-      <c r="W61" s="113"/>
+      <c r="O61" s="27"/>
+      <c r="P61" s="28"/>
+      <c r="Q61" s="28"/>
+      <c r="R61" s="29"/>
+      <c r="S61" s="27"/>
+      <c r="T61" s="28"/>
+      <c r="U61" s="29"/>
+      <c r="V61" s="25"/>
+      <c r="W61" s="26"/>
       <c r="X61" s="15"/>
       <c r="Y61" s="24"/>
       <c r="Z61" s="22"/>
       <c r="AA61" s="22"/>
     </row>
     <row r="62" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="83"/>
-      <c r="C62" s="84"/>
-      <c r="D62" s="84"/>
-      <c r="E62" s="85"/>
-      <c r="F62" s="83"/>
-      <c r="G62" s="84"/>
-      <c r="H62" s="85"/>
-      <c r="I62" s="112"/>
-      <c r="J62" s="113"/>
+      <c r="B62" s="27"/>
+      <c r="C62" s="28"/>
+      <c r="D62" s="28"/>
+      <c r="E62" s="29"/>
+      <c r="F62" s="27"/>
+      <c r="G62" s="28"/>
+      <c r="H62" s="29"/>
+      <c r="I62" s="25"/>
+      <c r="J62" s="26"/>
       <c r="K62" s="15"/>
       <c r="L62" s="22"/>
       <c r="M62" s="19"/>
       <c r="N62" s="23"/>
-      <c r="O62" s="91" t="s">
+      <c r="O62" s="55" t="s">
         <v>15</v>
       </c>
-      <c r="P62" s="92"/>
-      <c r="Q62" s="92"/>
-      <c r="R62" s="92"/>
-      <c r="S62" s="92"/>
-      <c r="T62" s="92"/>
-      <c r="U62" s="92"/>
-      <c r="V62" s="93"/>
-      <c r="W62" s="86" t="s">
+      <c r="P62" s="56"/>
+      <c r="Q62" s="56"/>
+      <c r="R62" s="56"/>
+      <c r="S62" s="56"/>
+      <c r="T62" s="56"/>
+      <c r="U62" s="56"/>
+      <c r="V62" s="57"/>
+      <c r="W62" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="X62" s="86"/>
-      <c r="Y62" s="86"/>
-      <c r="Z62" s="86" t="s">
+      <c r="X62" s="32"/>
+      <c r="Y62" s="32"/>
+      <c r="Z62" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="AA62" s="86"/>
+      <c r="AA62" s="32"/>
     </row>
     <row r="63" spans="2:27" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B63" s="83"/>
-      <c r="C63" s="84"/>
-      <c r="D63" s="84"/>
-      <c r="E63" s="85"/>
-      <c r="F63" s="83"/>
-      <c r="G63" s="84"/>
-      <c r="H63" s="85"/>
-      <c r="I63" s="112"/>
-      <c r="J63" s="113"/>
+      <c r="B63" s="27"/>
+      <c r="C63" s="28"/>
+      <c r="D63" s="28"/>
+      <c r="E63" s="29"/>
+      <c r="F63" s="27"/>
+      <c r="G63" s="28"/>
+      <c r="H63" s="29"/>
+      <c r="I63" s="25"/>
+      <c r="J63" s="26"/>
       <c r="K63" s="15"/>
       <c r="L63" s="22"/>
       <c r="M63" s="19"/>
       <c r="N63" s="23"/>
-      <c r="O63" s="94"/>
-      <c r="P63" s="95"/>
-      <c r="Q63" s="95"/>
-      <c r="R63" s="95"/>
-      <c r="S63" s="95"/>
-      <c r="T63" s="95"/>
-      <c r="U63" s="95"/>
-      <c r="V63" s="96"/>
-      <c r="W63" s="82"/>
-      <c r="X63" s="82"/>
-      <c r="Y63" s="82"/>
-      <c r="Z63" s="82"/>
-      <c r="AA63" s="82"/>
+      <c r="O63" s="58"/>
+      <c r="P63" s="59"/>
+      <c r="Q63" s="59"/>
+      <c r="R63" s="59"/>
+      <c r="S63" s="59"/>
+      <c r="T63" s="59"/>
+      <c r="U63" s="59"/>
+      <c r="V63" s="60"/>
+      <c r="W63" s="53"/>
+      <c r="X63" s="53"/>
+      <c r="Y63" s="53"/>
+      <c r="Z63" s="53"/>
+      <c r="AA63" s="53"/>
     </row>
     <row r="64" spans="2:27" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="65" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -10669,59 +10665,80 @@
     </row>
   </sheetData>
   <mergeCells count="151">
-    <mergeCell ref="V60:W60"/>
-    <mergeCell ref="V61:W61"/>
-    <mergeCell ref="I61:J61"/>
-    <mergeCell ref="I62:J62"/>
-    <mergeCell ref="I63:J63"/>
-    <mergeCell ref="B62:E62"/>
-    <mergeCell ref="F62:H62"/>
-    <mergeCell ref="B63:E63"/>
-    <mergeCell ref="F63:H63"/>
-    <mergeCell ref="O61:R61"/>
-    <mergeCell ref="S61:U61"/>
-    <mergeCell ref="O60:R60"/>
-    <mergeCell ref="S60:U60"/>
-    <mergeCell ref="I60:J60"/>
-    <mergeCell ref="F59:H59"/>
-    <mergeCell ref="F58:H58"/>
-    <mergeCell ref="B57:E57"/>
-    <mergeCell ref="F57:H57"/>
-    <mergeCell ref="B54:AA54"/>
-    <mergeCell ref="B58:E58"/>
-    <mergeCell ref="O56:R56"/>
-    <mergeCell ref="S56:U56"/>
-    <mergeCell ref="O57:R57"/>
-    <mergeCell ref="S57:U57"/>
-    <mergeCell ref="O58:R58"/>
-    <mergeCell ref="S58:U58"/>
-    <mergeCell ref="O59:R59"/>
-    <mergeCell ref="S59:U59"/>
-    <mergeCell ref="V56:W56"/>
-    <mergeCell ref="V57:W57"/>
-    <mergeCell ref="V58:W58"/>
-    <mergeCell ref="V59:W59"/>
-    <mergeCell ref="I56:J56"/>
-    <mergeCell ref="I57:J57"/>
-    <mergeCell ref="I58:J58"/>
-    <mergeCell ref="I59:J59"/>
-    <mergeCell ref="X42:Y42"/>
-    <mergeCell ref="X45:Y45"/>
-    <mergeCell ref="X48:Y48"/>
-    <mergeCell ref="L48:M48"/>
-    <mergeCell ref="B45:C47"/>
-    <mergeCell ref="R48:S48"/>
-    <mergeCell ref="B42:C44"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="H45:I45"/>
-    <mergeCell ref="J45:K45"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="L45:M45"/>
-    <mergeCell ref="B48:C53"/>
-    <mergeCell ref="P51:Q51"/>
-    <mergeCell ref="R51:S51"/>
-    <mergeCell ref="V51:W51"/>
-    <mergeCell ref="X51:Y51"/>
+    <mergeCell ref="B41:AA41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="N48:O48"/>
+    <mergeCell ref="P48:Q48"/>
+    <mergeCell ref="Z45:AA45"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="L42:M42"/>
+    <mergeCell ref="N42:O42"/>
+    <mergeCell ref="P42:Q42"/>
+    <mergeCell ref="R42:S42"/>
+    <mergeCell ref="Z42:AA42"/>
+    <mergeCell ref="N45:O45"/>
+    <mergeCell ref="P45:Q45"/>
+    <mergeCell ref="R45:S45"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="H48:I48"/>
+    <mergeCell ref="J48:K48"/>
+    <mergeCell ref="V42:W42"/>
+    <mergeCell ref="V45:W45"/>
+    <mergeCell ref="T42:U42"/>
+    <mergeCell ref="T45:U45"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="R34:V39"/>
+    <mergeCell ref="W34:AA39"/>
+    <mergeCell ref="B40:AA40"/>
+    <mergeCell ref="N12:R12"/>
+    <mergeCell ref="S10:U10"/>
+    <mergeCell ref="S11:U11"/>
+    <mergeCell ref="S12:U12"/>
+    <mergeCell ref="B17:Q17"/>
+    <mergeCell ref="B15:Q15"/>
+    <mergeCell ref="B16:Q16"/>
+    <mergeCell ref="B18:Q18"/>
+    <mergeCell ref="B13:AA13"/>
+    <mergeCell ref="B14:Q14"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="E10:J10"/>
+    <mergeCell ref="E11:J11"/>
+    <mergeCell ref="E12:J12"/>
+    <mergeCell ref="K10:M10"/>
+    <mergeCell ref="K12:M12"/>
+    <mergeCell ref="K11:M11"/>
+    <mergeCell ref="N10:R10"/>
+    <mergeCell ref="V10:AA10"/>
+    <mergeCell ref="V11:AA11"/>
+    <mergeCell ref="V12:AA12"/>
+    <mergeCell ref="B21:Q21"/>
+    <mergeCell ref="B22:Q39"/>
+    <mergeCell ref="R15:V21"/>
+    <mergeCell ref="W15:AA21"/>
+    <mergeCell ref="R22:V27"/>
+    <mergeCell ref="W22:AA27"/>
+    <mergeCell ref="R28:V33"/>
+    <mergeCell ref="N11:R11"/>
+    <mergeCell ref="R14:V14"/>
+    <mergeCell ref="W14:AA14"/>
+    <mergeCell ref="W28:AA33"/>
+    <mergeCell ref="B19:Q20"/>
+    <mergeCell ref="S2:U3"/>
+    <mergeCell ref="V2:X3"/>
+    <mergeCell ref="Y2:AA3"/>
+    <mergeCell ref="S4:U6"/>
+    <mergeCell ref="V4:X6"/>
+    <mergeCell ref="Y4:AA6"/>
+    <mergeCell ref="B6:R9"/>
+    <mergeCell ref="S8:U8"/>
+    <mergeCell ref="V8:AA8"/>
+    <mergeCell ref="S9:U9"/>
+    <mergeCell ref="V9:W9"/>
+    <mergeCell ref="Y9:Z9"/>
     <mergeCell ref="Z63:AA63"/>
     <mergeCell ref="Z48:AA48"/>
     <mergeCell ref="B61:E61"/>
@@ -10746,80 +10763,59 @@
     <mergeCell ref="V48:W48"/>
     <mergeCell ref="F56:H56"/>
     <mergeCell ref="B59:E59"/>
-    <mergeCell ref="S2:U3"/>
-    <mergeCell ref="V2:X3"/>
-    <mergeCell ref="Y2:AA3"/>
-    <mergeCell ref="S4:U6"/>
-    <mergeCell ref="V4:X6"/>
-    <mergeCell ref="Y4:AA6"/>
-    <mergeCell ref="B6:R9"/>
-    <mergeCell ref="S8:U8"/>
-    <mergeCell ref="V8:AA8"/>
-    <mergeCell ref="S9:U9"/>
-    <mergeCell ref="V9:W9"/>
-    <mergeCell ref="Y9:Z9"/>
-    <mergeCell ref="V11:AA11"/>
-    <mergeCell ref="V12:AA12"/>
-    <mergeCell ref="B21:Q21"/>
-    <mergeCell ref="B22:Q39"/>
-    <mergeCell ref="R15:V21"/>
-    <mergeCell ref="W15:AA21"/>
-    <mergeCell ref="R22:V27"/>
-    <mergeCell ref="W22:AA27"/>
-    <mergeCell ref="R28:V33"/>
-    <mergeCell ref="N11:R11"/>
-    <mergeCell ref="R14:V14"/>
-    <mergeCell ref="W14:AA14"/>
-    <mergeCell ref="W28:AA33"/>
-    <mergeCell ref="B19:Q20"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="R34:V39"/>
-    <mergeCell ref="W34:AA39"/>
-    <mergeCell ref="B40:AA40"/>
-    <mergeCell ref="N12:R12"/>
-    <mergeCell ref="S10:U10"/>
-    <mergeCell ref="S11:U11"/>
-    <mergeCell ref="S12:U12"/>
-    <mergeCell ref="B17:Q17"/>
-    <mergeCell ref="B15:Q15"/>
-    <mergeCell ref="B16:Q16"/>
-    <mergeCell ref="B18:Q18"/>
-    <mergeCell ref="B13:AA13"/>
-    <mergeCell ref="B14:Q14"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="E10:J10"/>
-    <mergeCell ref="E11:J11"/>
-    <mergeCell ref="E12:J12"/>
-    <mergeCell ref="K10:M10"/>
-    <mergeCell ref="K12:M12"/>
-    <mergeCell ref="K11:M11"/>
-    <mergeCell ref="N10:R10"/>
-    <mergeCell ref="V10:AA10"/>
-    <mergeCell ref="B41:AA41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="N48:O48"/>
-    <mergeCell ref="P48:Q48"/>
-    <mergeCell ref="Z45:AA45"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="J42:K42"/>
-    <mergeCell ref="L42:M42"/>
-    <mergeCell ref="N42:O42"/>
-    <mergeCell ref="P42:Q42"/>
-    <mergeCell ref="R42:S42"/>
-    <mergeCell ref="Z42:AA42"/>
-    <mergeCell ref="N45:O45"/>
-    <mergeCell ref="P45:Q45"/>
-    <mergeCell ref="R45:S45"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="H48:I48"/>
-    <mergeCell ref="J48:K48"/>
-    <mergeCell ref="V42:W42"/>
-    <mergeCell ref="V45:W45"/>
-    <mergeCell ref="T42:U42"/>
-    <mergeCell ref="T45:U45"/>
+    <mergeCell ref="X42:Y42"/>
+    <mergeCell ref="X45:Y45"/>
+    <mergeCell ref="X48:Y48"/>
+    <mergeCell ref="L48:M48"/>
+    <mergeCell ref="B45:C47"/>
+    <mergeCell ref="R48:S48"/>
+    <mergeCell ref="B42:C44"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="H45:I45"/>
+    <mergeCell ref="J45:K45"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="L45:M45"/>
+    <mergeCell ref="B48:C53"/>
+    <mergeCell ref="P51:Q51"/>
+    <mergeCell ref="R51:S51"/>
+    <mergeCell ref="V51:W51"/>
+    <mergeCell ref="X51:Y51"/>
+    <mergeCell ref="F59:H59"/>
+    <mergeCell ref="F58:H58"/>
+    <mergeCell ref="B57:E57"/>
+    <mergeCell ref="F57:H57"/>
+    <mergeCell ref="B54:AA54"/>
+    <mergeCell ref="B58:E58"/>
+    <mergeCell ref="O56:R56"/>
+    <mergeCell ref="S56:U56"/>
+    <mergeCell ref="O57:R57"/>
+    <mergeCell ref="S57:U57"/>
+    <mergeCell ref="O58:R58"/>
+    <mergeCell ref="S58:U58"/>
+    <mergeCell ref="O59:R59"/>
+    <mergeCell ref="S59:U59"/>
+    <mergeCell ref="V56:W56"/>
+    <mergeCell ref="V57:W57"/>
+    <mergeCell ref="V58:W58"/>
+    <mergeCell ref="V59:W59"/>
+    <mergeCell ref="I56:J56"/>
+    <mergeCell ref="I57:J57"/>
+    <mergeCell ref="I58:J58"/>
+    <mergeCell ref="I59:J59"/>
+    <mergeCell ref="V60:W60"/>
+    <mergeCell ref="V61:W61"/>
+    <mergeCell ref="I61:J61"/>
+    <mergeCell ref="I62:J62"/>
+    <mergeCell ref="I63:J63"/>
+    <mergeCell ref="B62:E62"/>
+    <mergeCell ref="F62:H62"/>
+    <mergeCell ref="B63:E63"/>
+    <mergeCell ref="F63:H63"/>
+    <mergeCell ref="O61:R61"/>
+    <mergeCell ref="S61:U61"/>
+    <mergeCell ref="O60:R60"/>
+    <mergeCell ref="S60:U60"/>
+    <mergeCell ref="I60:J60"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>